<commit_message>
Refresh dashboard data to 16 markets from query 16 prod run.
Add US-L/XL, CA-L/XL, DACH-S, and BNL-XL ideal HC coverage; optimize sql/16 by deriving market_accounts from rep_level.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/data/headcount-dashboard.xlsx
+++ b/docs/data/headcount-dashboard.xlsx
@@ -12,7 +12,7 @@
     <sheet name="About" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Markets'!$A$1:$AC$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Markets'!$A$1:$AC$17</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC11"/>
+  <dimension ref="A1:AC17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -644,7 +644,7 @@
         <v>80</v>
       </c>
       <c r="K2" t="n">
-        <v>0.187</v>
+        <v>0.188</v>
       </c>
       <c r="L2" t="n">
         <v>55</v>
@@ -653,7 +653,7 @@
         <v>40049</v>
       </c>
       <c r="N2" t="n">
-        <v>191378311</v>
+        <v>191378836</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -707,27 +707,27 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>UK-M</t>
+          <t>US-XL</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>UK</t>
+          <t>US</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>XL</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>1313</v>
+        <v>1296</v>
       </c>
       <c r="E3" t="n">
-        <v>160</v>
+        <v>906</v>
       </c>
       <c r="F3" t="n">
-        <v>-1153</v>
+        <v>-390</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -746,70 +746,33 @@
         <v>10</v>
       </c>
       <c r="K3" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="L3" t="n">
-        <v>41</v>
+        <v>7</v>
       </c>
       <c r="M3" t="n">
-        <v>6564</v>
+        <v>6482</v>
       </c>
       <c r="N3" t="n">
-        <v>22290790</v>
+        <v>122120633</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Hire + build books from SBS</t>
-        </is>
-      </c>
-      <c r="P3" t="n">
-        <v>47.9</v>
-      </c>
-      <c r="Q3" t="n">
-        <v>-0.056</v>
+          <t>Hire</t>
+        </is>
       </c>
       <c r="S3" t="n">
         <v>0</v>
       </c>
-      <c r="T3" t="n">
-        <v>17406</v>
-      </c>
-      <c r="U3" t="n">
-        <v>17062549</v>
-      </c>
       <c r="V3" t="n">
-        <v>3481</v>
-      </c>
-      <c r="W3" t="n">
-        <v>80</v>
-      </c>
-      <c r="X3" t="n">
-        <v>47.8</v>
-      </c>
-      <c r="Y3" t="inlineStr">
-        <is>
-          <t>Growing</t>
-        </is>
-      </c>
-      <c r="Z3" t="n">
-        <v>10</v>
-      </c>
-      <c r="AA3" t="n">
-        <v>10</v>
-      </c>
-      <c r="AB3" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC3" t="inlineStr">
-        <is>
-          <t>Declining</t>
-        </is>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>US-S</t>
+          <t>US-L</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -819,17 +782,17 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>L</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>118</v>
+        <v>480</v>
       </c>
       <c r="E4" t="n">
-        <v>508</v>
+        <v>785</v>
       </c>
       <c r="F4" t="n">
-        <v>390</v>
+        <v>305</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -837,86 +800,49 @@
         </is>
       </c>
       <c r="H4" t="n">
-        <v>45</v>
+        <v>25</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>05: 41-50</t>
+          <t>03: 21-30</t>
         </is>
       </c>
       <c r="J4" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="K4" t="n">
         <v>0.2</v>
       </c>
       <c r="L4" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="M4" t="n">
-        <v>5300</v>
+        <v>12000</v>
       </c>
       <c r="N4" t="n">
-        <v>13240721</v>
+        <v>84612173</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
           <t>Optimize HC</t>
         </is>
       </c>
-      <c r="P4" t="n">
-        <v>46.7</v>
-      </c>
-      <c r="Q4" t="n">
-        <v>-0.08400000000000001</v>
-      </c>
       <c r="S4" t="n">
-        <v>17780</v>
-      </c>
-      <c r="T4" t="n">
-        <v>1765233</v>
-      </c>
-      <c r="U4" t="n">
-        <v>502167251</v>
+        <v>7850</v>
       </c>
       <c r="V4" t="n">
-        <v>39227</v>
-      </c>
-      <c r="W4" t="n">
-        <v>10</v>
-      </c>
-      <c r="X4" t="n">
-        <v>194.28</v>
-      </c>
-      <c r="Y4" t="inlineStr">
-        <is>
-          <t>Plateaued</t>
-        </is>
-      </c>
-      <c r="Z4" t="n">
-        <v>10</v>
-      </c>
-      <c r="AA4" t="n">
-        <v>29</v>
-      </c>
-      <c r="AB4" t="n">
-        <v>20</v>
-      </c>
-      <c r="AC4" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>DACH-M</t>
+          <t>UK-M</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>DACH</t>
+          <t>UK</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -925,70 +851,70 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>78</v>
+        <v>1313</v>
       </c>
       <c r="E5" t="n">
-        <v>131</v>
+        <v>160</v>
       </c>
       <c r="F5" t="n">
-        <v>53</v>
+        <v>-1153</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Optimize</t>
+          <t>Hire</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>73</v>
+        <v>5</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>07: 66-80</t>
+          <t>01: 1-10</t>
         </is>
       </c>
       <c r="J5" t="n">
+        <v>10</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="L5" t="n">
+        <v>41</v>
+      </c>
+      <c r="M5" t="n">
+        <v>6564</v>
+      </c>
+      <c r="N5" t="n">
+        <v>22290790</v>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>Hire + build books from SBS</t>
+        </is>
+      </c>
+      <c r="P5" t="n">
+        <v>47.9</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>-0.056</v>
+      </c>
+      <c r="S5" t="n">
+        <v>0</v>
+      </c>
+      <c r="T5" t="n">
+        <v>17406</v>
+      </c>
+      <c r="U5" t="n">
+        <v>17062549</v>
+      </c>
+      <c r="V5" t="n">
+        <v>3481</v>
+      </c>
+      <c r="W5" t="n">
         <v>80</v>
       </c>
-      <c r="K5" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="L5" t="n">
-        <v>43</v>
-      </c>
-      <c r="M5" t="n">
-        <v>5668</v>
-      </c>
-      <c r="N5" t="n">
-        <v>9407809</v>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>Optimize HC</t>
-        </is>
-      </c>
-      <c r="P5" t="n">
-        <v>50</v>
-      </c>
-      <c r="Q5" t="n">
-        <v>0.005</v>
-      </c>
-      <c r="S5" t="n">
-        <v>3930</v>
-      </c>
-      <c r="T5" t="n">
-        <v>10886</v>
-      </c>
-      <c r="U5" t="n">
-        <v>6745421</v>
-      </c>
-      <c r="V5" t="n">
-        <v>149</v>
-      </c>
-      <c r="W5" t="n">
-        <v>65</v>
-      </c>
       <c r="X5" t="n">
-        <v>44.3</v>
+        <v>47.8</v>
       </c>
       <c r="Y5" t="inlineStr">
         <is>
@@ -999,10 +925,10 @@
         <v>10</v>
       </c>
       <c r="AA5" t="n">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="AB5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AC5" t="inlineStr">
         <is>
@@ -1013,27 +939,27 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>UK-L</t>
+          <t>US-S</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>UK</t>
+          <t>US</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>S</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>140</v>
+        <v>118</v>
       </c>
       <c r="E6" t="n">
-        <v>172</v>
+        <v>508</v>
       </c>
       <c r="F6" t="n">
-        <v>32</v>
+        <v>390</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -1041,81 +967,81 @@
         </is>
       </c>
       <c r="H6" t="n">
-        <v>15</v>
+        <v>45</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>02: 11-20</t>
+          <t>05: 41-50</t>
         </is>
       </c>
       <c r="J6" t="n">
+        <v>50</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="L6" t="n">
+        <v>10</v>
+      </c>
+      <c r="M6" t="n">
+        <v>5300</v>
+      </c>
+      <c r="N6" t="n">
+        <v>13240721</v>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>Optimize HC</t>
+        </is>
+      </c>
+      <c r="P6" t="n">
+        <v>46.7</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>-0.08400000000000001</v>
+      </c>
+      <c r="S6" t="n">
+        <v>17780</v>
+      </c>
+      <c r="T6" t="n">
+        <v>1765233</v>
+      </c>
+      <c r="U6" t="n">
+        <v>502167251</v>
+      </c>
+      <c r="V6" t="n">
+        <v>39227</v>
+      </c>
+      <c r="W6" t="n">
+        <v>10</v>
+      </c>
+      <c r="X6" t="n">
+        <v>194.28</v>
+      </c>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>Plateaued</t>
+        </is>
+      </c>
+      <c r="Z6" t="n">
+        <v>10</v>
+      </c>
+      <c r="AA6" t="n">
+        <v>29</v>
+      </c>
+      <c r="AB6" t="n">
         <v>20</v>
       </c>
-      <c r="K6" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="L6" t="n">
-        <v>12</v>
-      </c>
-      <c r="M6" t="n">
-        <v>2097</v>
-      </c>
-      <c r="N6" t="n">
-        <v>8301713</v>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>Optimize HC</t>
-        </is>
-      </c>
-      <c r="P6" t="n">
-        <v>49.9</v>
-      </c>
-      <c r="Q6" t="n">
-        <v>-0.014</v>
-      </c>
-      <c r="S6" t="n">
-        <v>516</v>
-      </c>
-      <c r="T6" t="n">
-        <v>1879</v>
-      </c>
-      <c r="U6" t="n">
-        <v>428831</v>
-      </c>
-      <c r="V6" t="n">
-        <v>125</v>
-      </c>
-      <c r="W6" t="n">
-        <v>20</v>
-      </c>
-      <c r="X6" t="n">
-        <v>7.2</v>
-      </c>
-      <c r="Y6" t="inlineStr">
-        <is>
-          <t>Growing</t>
-        </is>
-      </c>
-      <c r="Z6" t="n">
-        <v>10</v>
-      </c>
-      <c r="AA6" t="n">
-        <v>11</v>
-      </c>
-      <c r="AB6" t="n">
-        <v>5</v>
-      </c>
       <c r="AC6" t="inlineStr">
         <is>
-          <t>Declining</t>
+          <t>OK</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>DACH-L</t>
+          <t>DACH-M</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1125,104 +1051,104 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>M</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>401</v>
+        <v>78</v>
       </c>
       <c r="E7" t="n">
-        <v>154</v>
+        <v>131</v>
       </c>
       <c r="F7" t="n">
-        <v>-247</v>
+        <v>53</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Hire</t>
+          <t>Optimize</t>
         </is>
       </c>
       <c r="H7" t="n">
-        <v>5</v>
+        <v>73</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>01: 1-10</t>
+          <t>07: 66-80</t>
         </is>
       </c>
       <c r="J7" t="n">
-        <v>10</v>
+        <v>80</v>
       </c>
       <c r="K7" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="L7" t="n">
-        <v>13</v>
+        <v>43</v>
       </c>
       <c r="M7" t="n">
-        <v>2004</v>
+        <v>5669</v>
       </c>
       <c r="N7" t="n">
-        <v>4096268</v>
+        <v>9407836</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>Hire + build books from SBS</t>
+          <t>Optimize HC</t>
         </is>
       </c>
       <c r="P7" t="n">
-        <v>52.8</v>
+        <v>50</v>
       </c>
       <c r="Q7" t="n">
-        <v>0.055</v>
+        <v>0.005</v>
       </c>
       <c r="S7" t="n">
-        <v>0</v>
+        <v>3930</v>
       </c>
       <c r="T7" t="n">
-        <v>1298</v>
+        <v>10886</v>
       </c>
       <c r="U7" t="n">
-        <v>417037</v>
+        <v>6745421</v>
       </c>
       <c r="V7" t="n">
-        <v>259</v>
+        <v>149</v>
       </c>
       <c r="W7" t="n">
-        <v>10</v>
+        <v>65</v>
       </c>
       <c r="X7" t="n">
-        <v>10.8</v>
+        <v>44.3</v>
       </c>
       <c r="Y7" t="inlineStr">
         <is>
-          <t>Plateaued</t>
+          <t>Growing</t>
         </is>
       </c>
       <c r="Z7" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="AA7" t="n">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="AB7" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="AC7" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>Declining</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>BNL-L</t>
+          <t>UK-L</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>BNL</t>
+          <t>UK</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1231,13 +1157,13 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>66</v>
+        <v>140</v>
       </c>
       <c r="E8" t="n">
-        <v>88</v>
+        <v>172</v>
       </c>
       <c r="F8" t="n">
-        <v>22</v>
+        <v>32</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -1259,13 +1185,13 @@
         <v>0.3</v>
       </c>
       <c r="L8" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="M8" t="n">
-        <v>996</v>
+        <v>2097</v>
       </c>
       <c r="N8" t="n">
-        <v>2450421</v>
+        <v>8301713</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
@@ -1273,28 +1199,28 @@
         </is>
       </c>
       <c r="P8" t="n">
-        <v>49.8</v>
+        <v>49.9</v>
       </c>
       <c r="Q8" t="n">
-        <v>-0.022</v>
+        <v>-0.014</v>
       </c>
       <c r="S8" t="n">
-        <v>352</v>
+        <v>516</v>
       </c>
       <c r="T8" t="n">
-        <v>599</v>
+        <v>1879</v>
       </c>
       <c r="U8" t="n">
-        <v>351367</v>
+        <v>428831</v>
       </c>
       <c r="V8" t="n">
-        <v>39</v>
+        <v>125</v>
       </c>
       <c r="W8" t="n">
         <v>20</v>
       </c>
       <c r="X8" t="n">
-        <v>8.6</v>
+        <v>7.2</v>
       </c>
       <c r="Y8" t="inlineStr">
         <is>
@@ -1302,29 +1228,29 @@
         </is>
       </c>
       <c r="Z8" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="AA8" t="n">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="AB8" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AC8" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>Declining</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>FR-XL</t>
+          <t>CA-XL</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1333,13 +1259,13 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="E9" t="n">
-        <v>77</v>
+        <v>92</v>
       </c>
       <c r="F9" t="n">
-        <v>-39</v>
+        <v>-22</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -1361,87 +1287,50 @@
         <v>0.3</v>
       </c>
       <c r="L9" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="M9" t="n">
-        <v>582</v>
+        <v>569</v>
       </c>
       <c r="N9" t="n">
-        <v>1995476</v>
+        <v>4126601</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>Hire + build books from SBS</t>
-        </is>
-      </c>
-      <c r="P9" t="n">
-        <v>52.1</v>
-      </c>
-      <c r="Q9" t="n">
-        <v>0.032</v>
+          <t>Hire</t>
+        </is>
       </c>
       <c r="S9" t="n">
         <v>0</v>
       </c>
-      <c r="T9" t="n">
-        <v>637</v>
-      </c>
-      <c r="U9" t="n">
-        <v>80994</v>
-      </c>
       <c r="V9" t="n">
-        <v>127</v>
-      </c>
-      <c r="W9" t="n">
-        <v>10</v>
-      </c>
-      <c r="X9" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="Y9" t="inlineStr">
-        <is>
-          <t>Growing</t>
-        </is>
-      </c>
-      <c r="Z9" t="n">
-        <v>10</v>
-      </c>
-      <c r="AA9" t="n">
-        <v>6</v>
-      </c>
-      <c r="AB9" t="n">
-        <v>5</v>
-      </c>
-      <c r="AC9" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>UK-S</t>
+          <t>DACH-L</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>UK</t>
+          <t>DACH</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>L</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>368</v>
+        <v>401</v>
       </c>
       <c r="E10" t="n">
-        <v>141</v>
+        <v>154</v>
       </c>
       <c r="F10" t="n">
-        <v>-227</v>
+        <v>-247</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -1460,16 +1349,16 @@
         <v>10</v>
       </c>
       <c r="K10" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="L10" t="n">
         <v>13</v>
       </c>
       <c r="M10" t="n">
-        <v>1838</v>
+        <v>2004</v>
       </c>
       <c r="N10" t="n">
-        <v>974670</v>
+        <v>4096268</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
@@ -1477,28 +1366,28 @@
         </is>
       </c>
       <c r="P10" t="n">
-        <v>48.2</v>
+        <v>52.8</v>
       </c>
       <c r="Q10" t="n">
-        <v>-0.048</v>
+        <v>0.055</v>
       </c>
       <c r="S10" t="n">
         <v>0</v>
       </c>
       <c r="T10" t="n">
-        <v>364298</v>
+        <v>1298</v>
       </c>
       <c r="U10" t="n">
-        <v>53614691</v>
+        <v>417037</v>
       </c>
       <c r="V10" t="n">
-        <v>72859</v>
+        <v>259</v>
       </c>
       <c r="W10" t="n">
         <v>10</v>
       </c>
       <c r="X10" t="n">
-        <v>131.6</v>
+        <v>10.8</v>
       </c>
       <c r="Y10" t="inlineStr">
         <is>
@@ -1506,24 +1395,24 @@
         </is>
       </c>
       <c r="Z10" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="AA10" t="n">
-        <v>29</v>
+        <v>11</v>
       </c>
       <c r="AB10" t="n">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="AC10" t="inlineStr">
         <is>
-          <t>Declining</t>
+          <t>OK</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CA-S</t>
+          <t>CA-L</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1533,17 +1422,17 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>L</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>111</v>
+        <v>192</v>
       </c>
       <c r="E11" t="n">
-        <v>66</v>
+        <v>92</v>
       </c>
       <c r="F11" t="n">
-        <v>-45</v>
+        <v>-100</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -1562,68 +1451,569 @@
         <v>10</v>
       </c>
       <c r="K11" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="L11" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="M11" t="n">
-        <v>556</v>
+        <v>960</v>
       </c>
       <c r="N11" t="n">
-        <v>554640</v>
+        <v>3188432</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>Hire + build books from SBS</t>
-        </is>
-      </c>
-      <c r="P11" t="n">
-        <v>50</v>
-      </c>
-      <c r="Q11" t="n">
-        <v>-0.006</v>
+          <t>Hire</t>
+        </is>
       </c>
       <c r="S11" t="n">
         <v>0</v>
       </c>
-      <c r="T11" t="n">
+      <c r="V11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>BNL-XL</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>BNL</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>XL</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>101</v>
+      </c>
+      <c r="E12" t="n">
+        <v>88</v>
+      </c>
+      <c r="F12" t="n">
+        <v>-13</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Hire</t>
+        </is>
+      </c>
+      <c r="H12" t="n">
+        <v>5</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>01: 1-10</t>
+        </is>
+      </c>
+      <c r="J12" t="n">
+        <v>10</v>
+      </c>
+      <c r="K12" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="L12" t="n">
+        <v>6</v>
+      </c>
+      <c r="M12" t="n">
+        <v>505</v>
+      </c>
+      <c r="N12" t="n">
+        <v>2748456</v>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>Hire</t>
+        </is>
+      </c>
+      <c r="S12" t="n">
+        <v>0</v>
+      </c>
+      <c r="V12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>BNL-L</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>BNL</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>66</v>
+      </c>
+      <c r="E13" t="n">
+        <v>88</v>
+      </c>
+      <c r="F13" t="n">
+        <v>22</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Optimize</t>
+        </is>
+      </c>
+      <c r="H13" t="n">
+        <v>15</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>02: 11-20</t>
+        </is>
+      </c>
+      <c r="J13" t="n">
+        <v>20</v>
+      </c>
+      <c r="K13" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="L13" t="n">
+        <v>11</v>
+      </c>
+      <c r="M13" t="n">
+        <v>996</v>
+      </c>
+      <c r="N13" t="n">
+        <v>2450421</v>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>Optimize HC</t>
+        </is>
+      </c>
+      <c r="P13" t="n">
+        <v>49.8</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>-0.022</v>
+      </c>
+      <c r="S13" t="n">
+        <v>352</v>
+      </c>
+      <c r="T13" t="n">
+        <v>599</v>
+      </c>
+      <c r="U13" t="n">
+        <v>351367</v>
+      </c>
+      <c r="V13" t="n">
+        <v>39</v>
+      </c>
+      <c r="W13" t="n">
+        <v>20</v>
+      </c>
+      <c r="X13" t="n">
+        <v>8.6</v>
+      </c>
+      <c r="Y13" t="inlineStr">
+        <is>
+          <t>Growing</t>
+        </is>
+      </c>
+      <c r="Z13" t="n">
+        <v>20</v>
+      </c>
+      <c r="AA13" t="n">
+        <v>17</v>
+      </c>
+      <c r="AB13" t="n">
+        <v>6</v>
+      </c>
+      <c r="AC13" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>FR-XL</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>XL</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>116</v>
+      </c>
+      <c r="E14" t="n">
+        <v>77</v>
+      </c>
+      <c r="F14" t="n">
+        <v>-39</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Hire</t>
+        </is>
+      </c>
+      <c r="H14" t="n">
+        <v>5</v>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>01: 1-10</t>
+        </is>
+      </c>
+      <c r="J14" t="n">
+        <v>10</v>
+      </c>
+      <c r="K14" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="L14" t="n">
+        <v>8</v>
+      </c>
+      <c r="M14" t="n">
+        <v>582</v>
+      </c>
+      <c r="N14" t="n">
+        <v>1995476</v>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>Hire + build books from SBS</t>
+        </is>
+      </c>
+      <c r="P14" t="n">
+        <v>52.1</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>0.032</v>
+      </c>
+      <c r="S14" t="n">
+        <v>0</v>
+      </c>
+      <c r="T14" t="n">
+        <v>637</v>
+      </c>
+      <c r="U14" t="n">
+        <v>80994</v>
+      </c>
+      <c r="V14" t="n">
+        <v>127</v>
+      </c>
+      <c r="W14" t="n">
+        <v>10</v>
+      </c>
+      <c r="X14" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="Y14" t="inlineStr">
+        <is>
+          <t>Growing</t>
+        </is>
+      </c>
+      <c r="Z14" t="n">
+        <v>10</v>
+      </c>
+      <c r="AA14" t="n">
+        <v>6</v>
+      </c>
+      <c r="AB14" t="n">
+        <v>5</v>
+      </c>
+      <c r="AC14" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>DACH-S</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>DACH</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>403</v>
+      </c>
+      <c r="E15" t="n">
+        <v>122</v>
+      </c>
+      <c r="F15" t="n">
+        <v>-281</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Hire</t>
+        </is>
+      </c>
+      <c r="H15" t="n">
+        <v>5</v>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>01: 1-10</t>
+        </is>
+      </c>
+      <c r="J15" t="n">
+        <v>10</v>
+      </c>
+      <c r="K15" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="L15" t="n">
+        <v>17</v>
+      </c>
+      <c r="M15" t="n">
+        <v>2017</v>
+      </c>
+      <c r="N15" t="n">
+        <v>1171728</v>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>Hire</t>
+        </is>
+      </c>
+      <c r="S15" t="n">
+        <v>0</v>
+      </c>
+      <c r="V15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>UK-S</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>368</v>
+      </c>
+      <c r="E16" t="n">
+        <v>141</v>
+      </c>
+      <c r="F16" t="n">
+        <v>-227</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Hire</t>
+        </is>
+      </c>
+      <c r="H16" t="n">
+        <v>5</v>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>01: 1-10</t>
+        </is>
+      </c>
+      <c r="J16" t="n">
+        <v>10</v>
+      </c>
+      <c r="K16" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="L16" t="n">
+        <v>13</v>
+      </c>
+      <c r="M16" t="n">
+        <v>1839</v>
+      </c>
+      <c r="N16" t="n">
+        <v>974670</v>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>Hire + build books from SBS</t>
+        </is>
+      </c>
+      <c r="P16" t="n">
+        <v>48.2</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>-0.048</v>
+      </c>
+      <c r="S16" t="n">
+        <v>0</v>
+      </c>
+      <c r="T16" t="n">
+        <v>364298</v>
+      </c>
+      <c r="U16" t="n">
+        <v>53614691</v>
+      </c>
+      <c r="V16" t="n">
+        <v>72859</v>
+      </c>
+      <c r="W16" t="n">
+        <v>10</v>
+      </c>
+      <c r="X16" t="n">
+        <v>131.6</v>
+      </c>
+      <c r="Y16" t="inlineStr">
+        <is>
+          <t>Plateaued</t>
+        </is>
+      </c>
+      <c r="Z16" t="n">
+        <v>10</v>
+      </c>
+      <c r="AA16" t="n">
+        <v>29</v>
+      </c>
+      <c r="AB16" t="n">
+        <v>20</v>
+      </c>
+      <c r="AC16" t="inlineStr">
+        <is>
+          <t>Declining</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>CA-S</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>111</v>
+      </c>
+      <c r="E17" t="n">
+        <v>66</v>
+      </c>
+      <c r="F17" t="n">
+        <v>-45</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Hire</t>
+        </is>
+      </c>
+      <c r="H17" t="n">
+        <v>5</v>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>01: 1-10</t>
+        </is>
+      </c>
+      <c r="J17" t="n">
+        <v>10</v>
+      </c>
+      <c r="K17" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="L17" t="n">
+        <v>8</v>
+      </c>
+      <c r="M17" t="n">
+        <v>556</v>
+      </c>
+      <c r="N17" t="n">
+        <v>554640</v>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>Hire + build books from SBS</t>
+        </is>
+      </c>
+      <c r="P17" t="n">
+        <v>50</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>-0.006</v>
+      </c>
+      <c r="S17" t="n">
+        <v>0</v>
+      </c>
+      <c r="T17" t="n">
         <v>276061</v>
       </c>
-      <c r="U11" t="n">
+      <c r="U17" t="n">
         <v>41707962</v>
       </c>
-      <c r="V11" t="n">
+      <c r="V17" t="n">
         <v>55212</v>
       </c>
-      <c r="W11" t="n">
-        <v>10</v>
-      </c>
-      <c r="X11" t="n">
+      <c r="W17" t="n">
+        <v>10</v>
+      </c>
+      <c r="X17" t="n">
         <v>93.8</v>
       </c>
-      <c r="Y11" t="inlineStr">
+      <c r="Y17" t="inlineStr">
         <is>
           <t>Growing</t>
         </is>
       </c>
-      <c r="Z11" t="n">
-        <v>10</v>
-      </c>
-      <c r="AA11" t="n">
+      <c r="Z17" t="n">
+        <v>10</v>
+      </c>
+      <c r="AA17" t="n">
         <v>20</v>
       </c>
-      <c r="AB11" t="n">
+      <c r="AB17" t="n">
         <v>20</v>
       </c>
-      <c r="AC11" t="inlineStr">
+      <c r="AC17" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AC11"/>
+  <autoFilter ref="A1:AC17"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add Layer 1 book health and Layer 2 book action to dashboard.
Extend sql/16 with PQR, ideal PCID, too-big/too-little counts, and split-hire; add sql/17 rep flags, lookup UX, and book health/action panels.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/data/headcount-dashboard.xlsx
+++ b/docs/data/headcount-dashboard.xlsx
@@ -12,7 +12,7 @@
     <sheet name="About" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Markets'!$A$1:$AC$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Markets'!$A$1:$AN$17</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -421,38 +421,49 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC17"/>
+  <dimension ref="A1:AN17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="17" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="19" customWidth="1" min="7" max="7"/>
-    <col width="32" customWidth="1" min="8" max="8"/>
-    <col width="21" customWidth="1" min="9" max="9"/>
-    <col width="22" customWidth="1" min="10" max="10"/>
-    <col width="23" customWidth="1" min="11" max="11"/>
-    <col width="18" customWidth="1" min="12" max="12"/>
-    <col width="19" customWidth="1" min="13" max="13"/>
+    <col width="27" customWidth="1" min="5" max="5"/>
+    <col width="21" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="19" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
     <col width="17" customWidth="1" min="14" max="14"/>
-    <col width="20" customWidth="1" min="15" max="15"/>
-    <col width="19" customWidth="1" min="16" max="16"/>
-    <col width="17" customWidth="1" min="17" max="17"/>
-    <col width="21" customWidth="1" min="18" max="18"/>
-    <col width="19" customWidth="1" min="19" max="19"/>
-    <col width="26" customWidth="1" min="20" max="20"/>
-    <col width="21" customWidth="1" min="21" max="21"/>
-    <col width="26" customWidth="1" min="22" max="22"/>
-    <col width="22" customWidth="1" min="23" max="23"/>
+    <col width="22" customWidth="1" min="15" max="15"/>
+    <col width="22" customWidth="1" min="16" max="16"/>
+    <col width="23" customWidth="1" min="17" max="17"/>
+    <col width="24" customWidth="1" min="18" max="18"/>
+    <col width="32" customWidth="1" min="19" max="19"/>
+    <col width="21" customWidth="1" min="20" max="20"/>
+    <col width="22" customWidth="1" min="21" max="21"/>
+    <col width="23" customWidth="1" min="22" max="22"/>
+    <col width="18" customWidth="1" min="23" max="23"/>
     <col width="19" customWidth="1" min="24" max="24"/>
-    <col width="21" customWidth="1" min="25" max="25"/>
-    <col width="30" customWidth="1" min="26" max="26"/>
-    <col width="24" customWidth="1" min="27" max="27"/>
-    <col width="29" customWidth="1" min="28" max="28"/>
-    <col width="17" customWidth="1" min="29" max="29"/>
+    <col width="17" customWidth="1" min="25" max="25"/>
+    <col width="20" customWidth="1" min="26" max="26"/>
+    <col width="19" customWidth="1" min="27" max="27"/>
+    <col width="17" customWidth="1" min="28" max="28"/>
+    <col width="21" customWidth="1" min="29" max="29"/>
+    <col width="19" customWidth="1" min="30" max="30"/>
+    <col width="26" customWidth="1" min="31" max="31"/>
+    <col width="21" customWidth="1" min="32" max="32"/>
+    <col width="26" customWidth="1" min="33" max="33"/>
+    <col width="22" customWidth="1" min="34" max="34"/>
+    <col width="19" customWidth="1" min="35" max="35"/>
+    <col width="21" customWidth="1" min="36" max="36"/>
+    <col width="30" customWidth="1" min="37" max="37"/>
+    <col width="24" customWidth="1" min="38" max="38"/>
+    <col width="29" customWidth="1" min="39" max="39"/>
+    <col width="17" customWidth="1" min="40" max="40"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -478,125 +489,180 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>Ideal PCID (accounts/rep)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Avg PQR per rep ($)</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Market PQR 90d ($)</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Rev vs PQR %</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
           <t>Current reps</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Avg PCID per rep</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Headcount gap</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>HC recommendation</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Reps too big</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Reps too little</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Splittable PCID pool</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>New heads from split</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Book action (Layer 2)</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>Split hire recommended</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Ideal book size (accounts/rep)</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Perfect book bucket</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Perfect book ceiling</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Perfect book growth %</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>Current avg book</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>Assigned accounts</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>Revenue 90d ($)</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>Recommended action</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>FY26 % book built</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>FY26 book score</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>FY26 target % (TBD)</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>Headroom accounts</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>SBS whitespace (country)</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>SBS revenue 90d ($)</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>Books buildable from SBS</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="AH1" s="1" t="inlineStr">
         <is>
           <t>Opp plateau book max</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="AI1" s="1" t="inlineStr">
         <is>
           <t>Opp plateau $/job</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="AJ1" s="1" t="inlineStr">
         <is>
           <t>Opp pipeline status</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="AK1" s="1" t="inlineStr">
         <is>
           <t>Coverage inflection book max</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AL1" s="1" t="inlineStr">
         <is>
           <t>Coverage at inflection</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AM1" s="1" t="inlineStr">
         <is>
           <t>Median impact calls/account</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AN1" s="1" t="inlineStr">
         <is>
           <t>Coverage status</t>
         </is>
@@ -622,83 +688,89 @@
         <v>549</v>
       </c>
       <c r="E2" t="n">
+        <v>73</v>
+      </c>
+      <c r="I2" t="n">
         <v>735</v>
       </c>
-      <c r="F2" t="n">
+      <c r="J2" t="n">
+        <v>55</v>
+      </c>
+      <c r="K2" t="n">
         <v>186</v>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>Optimize</t>
         </is>
       </c>
-      <c r="H2" t="n">
+      <c r="S2" t="n">
         <v>73</v>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="T2" t="inlineStr">
         <is>
           <t>07: 66-80</t>
         </is>
       </c>
-      <c r="J2" t="n">
+      <c r="U2" t="n">
         <v>80</v>
       </c>
-      <c r="K2" t="n">
+      <c r="V2" t="n">
         <v>0.188</v>
       </c>
-      <c r="L2" t="n">
+      <c r="W2" t="n">
         <v>55</v>
       </c>
-      <c r="M2" t="n">
+      <c r="X2" t="n">
         <v>40049</v>
       </c>
-      <c r="N2" t="n">
+      <c r="Y2" t="n">
         <v>191378836</v>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="Z2" t="inlineStr">
         <is>
           <t>Optimize HC</t>
         </is>
       </c>
-      <c r="P2" t="n">
+      <c r="AA2" t="n">
         <v>46.9</v>
       </c>
-      <c r="Q2" t="n">
+      <c r="AB2" t="n">
         <v>-0.076</v>
       </c>
-      <c r="S2" t="n">
+      <c r="AD2" t="n">
         <v>13230</v>
       </c>
-      <c r="T2" t="n">
+      <c r="AE2" t="n">
         <v>103681</v>
       </c>
-      <c r="U2" t="n">
+      <c r="AF2" t="n">
         <v>160679658</v>
       </c>
-      <c r="V2" t="n">
+      <c r="AG2" t="n">
         <v>1420</v>
       </c>
-      <c r="W2" t="n">
+      <c r="AH2" t="n">
         <v>100</v>
       </c>
-      <c r="X2" t="n">
+      <c r="AI2" t="n">
         <v>61.96</v>
       </c>
-      <c r="Y2" t="inlineStr">
+      <c r="AJ2" t="inlineStr">
         <is>
           <t>Growing</t>
         </is>
       </c>
-      <c r="Z2" t="n">
-        <v>10</v>
-      </c>
-      <c r="AA2" t="n">
+      <c r="AK2" t="n">
+        <v>10</v>
+      </c>
+      <c r="AL2" t="n">
         <v>15</v>
       </c>
-      <c r="AB2" t="n">
+      <c r="AM2" t="n">
         <v>1</v>
       </c>
-      <c r="AC2" t="inlineStr">
+      <c r="AN2" t="inlineStr">
         <is>
           <t>Declining</t>
         </is>
@@ -724,48 +796,54 @@
         <v>1296</v>
       </c>
       <c r="E3" t="n">
+        <v>5</v>
+      </c>
+      <c r="I3" t="n">
         <v>906</v>
       </c>
-      <c r="F3" t="n">
+      <c r="J3" t="n">
+        <v>7</v>
+      </c>
+      <c r="K3" t="n">
         <v>-390</v>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>Hire</t>
         </is>
       </c>
-      <c r="H3" t="n">
+      <c r="S3" t="n">
         <v>5</v>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="T3" t="inlineStr">
         <is>
           <t>01: 1-10</t>
         </is>
       </c>
-      <c r="J3" t="n">
-        <v>10</v>
-      </c>
-      <c r="K3" t="n">
+      <c r="U3" t="n">
+        <v>10</v>
+      </c>
+      <c r="V3" t="n">
         <v>0.2</v>
       </c>
-      <c r="L3" t="n">
+      <c r="W3" t="n">
         <v>7</v>
       </c>
-      <c r="M3" t="n">
+      <c r="X3" t="n">
         <v>6482</v>
       </c>
-      <c r="N3" t="n">
+      <c r="Y3" t="n">
         <v>122120633</v>
       </c>
-      <c r="O3" t="inlineStr">
+      <c r="Z3" t="inlineStr">
         <is>
           <t>Hire</t>
         </is>
       </c>
-      <c r="S3" t="n">
+      <c r="AD3" t="n">
         <v>0</v>
       </c>
-      <c r="V3" t="n">
+      <c r="AG3" t="n">
         <v>0</v>
       </c>
     </row>
@@ -789,48 +867,54 @@
         <v>480</v>
       </c>
       <c r="E4" t="n">
+        <v>25</v>
+      </c>
+      <c r="I4" t="n">
         <v>785</v>
       </c>
-      <c r="F4" t="n">
+      <c r="J4" t="n">
+        <v>15</v>
+      </c>
+      <c r="K4" t="n">
         <v>305</v>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>Optimize</t>
         </is>
       </c>
-      <c r="H4" t="n">
+      <c r="S4" t="n">
         <v>25</v>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="T4" t="inlineStr">
         <is>
           <t>03: 21-30</t>
         </is>
       </c>
-      <c r="J4" t="n">
+      <c r="U4" t="n">
         <v>30</v>
       </c>
-      <c r="K4" t="n">
+      <c r="V4" t="n">
         <v>0.2</v>
       </c>
-      <c r="L4" t="n">
+      <c r="W4" t="n">
         <v>15</v>
       </c>
-      <c r="M4" t="n">
+      <c r="X4" t="n">
         <v>12000</v>
       </c>
-      <c r="N4" t="n">
+      <c r="Y4" t="n">
         <v>84612173</v>
       </c>
-      <c r="O4" t="inlineStr">
+      <c r="Z4" t="inlineStr">
         <is>
           <t>Optimize HC</t>
         </is>
       </c>
-      <c r="S4" t="n">
+      <c r="AD4" t="n">
         <v>7850</v>
       </c>
-      <c r="V4" t="n">
+      <c r="AG4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -854,83 +938,89 @@
         <v>1313</v>
       </c>
       <c r="E5" t="n">
+        <v>5</v>
+      </c>
+      <c r="I5" t="n">
         <v>160</v>
       </c>
-      <c r="F5" t="n">
+      <c r="J5" t="n">
+        <v>41</v>
+      </c>
+      <c r="K5" t="n">
         <v>-1153</v>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="L5" t="inlineStr">
         <is>
           <t>Hire</t>
         </is>
       </c>
-      <c r="H5" t="n">
+      <c r="S5" t="n">
         <v>5</v>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="T5" t="inlineStr">
         <is>
           <t>01: 1-10</t>
         </is>
       </c>
-      <c r="J5" t="n">
-        <v>10</v>
-      </c>
-      <c r="K5" t="n">
+      <c r="U5" t="n">
+        <v>10</v>
+      </c>
+      <c r="V5" t="n">
         <v>0.4</v>
       </c>
-      <c r="L5" t="n">
+      <c r="W5" t="n">
         <v>41</v>
       </c>
-      <c r="M5" t="n">
+      <c r="X5" t="n">
         <v>6564</v>
       </c>
-      <c r="N5" t="n">
+      <c r="Y5" t="n">
         <v>22290790</v>
       </c>
-      <c r="O5" t="inlineStr">
+      <c r="Z5" t="inlineStr">
         <is>
           <t>Hire + build books from SBS</t>
         </is>
       </c>
-      <c r="P5" t="n">
+      <c r="AA5" t="n">
         <v>47.9</v>
       </c>
-      <c r="Q5" t="n">
+      <c r="AB5" t="n">
         <v>-0.056</v>
       </c>
-      <c r="S5" t="n">
+      <c r="AD5" t="n">
         <v>0</v>
       </c>
-      <c r="T5" t="n">
+      <c r="AE5" t="n">
         <v>17406</v>
       </c>
-      <c r="U5" t="n">
+      <c r="AF5" t="n">
         <v>17062549</v>
       </c>
-      <c r="V5" t="n">
+      <c r="AG5" t="n">
         <v>3481</v>
       </c>
-      <c r="W5" t="n">
+      <c r="AH5" t="n">
         <v>80</v>
       </c>
-      <c r="X5" t="n">
+      <c r="AI5" t="n">
         <v>47.8</v>
       </c>
-      <c r="Y5" t="inlineStr">
+      <c r="AJ5" t="inlineStr">
         <is>
           <t>Growing</t>
         </is>
       </c>
-      <c r="Z5" t="n">
-        <v>10</v>
-      </c>
-      <c r="AA5" t="n">
-        <v>10</v>
-      </c>
-      <c r="AB5" t="n">
+      <c r="AK5" t="n">
+        <v>10</v>
+      </c>
+      <c r="AL5" t="n">
+        <v>10</v>
+      </c>
+      <c r="AM5" t="n">
         <v>1</v>
       </c>
-      <c r="AC5" t="inlineStr">
+      <c r="AN5" t="inlineStr">
         <is>
           <t>Declining</t>
         </is>
@@ -956,83 +1046,89 @@
         <v>118</v>
       </c>
       <c r="E6" t="n">
+        <v>45</v>
+      </c>
+      <c r="I6" t="n">
         <v>508</v>
       </c>
-      <c r="F6" t="n">
+      <c r="J6" t="n">
+        <v>10</v>
+      </c>
+      <c r="K6" t="n">
         <v>390</v>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="L6" t="inlineStr">
         <is>
           <t>Optimize</t>
         </is>
       </c>
-      <c r="H6" t="n">
+      <c r="S6" t="n">
         <v>45</v>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="T6" t="inlineStr">
         <is>
           <t>05: 41-50</t>
         </is>
       </c>
-      <c r="J6" t="n">
+      <c r="U6" t="n">
         <v>50</v>
       </c>
-      <c r="K6" t="n">
+      <c r="V6" t="n">
         <v>0.2</v>
       </c>
-      <c r="L6" t="n">
-        <v>10</v>
-      </c>
-      <c r="M6" t="n">
+      <c r="W6" t="n">
+        <v>10</v>
+      </c>
+      <c r="X6" t="n">
         <v>5300</v>
       </c>
-      <c r="N6" t="n">
+      <c r="Y6" t="n">
         <v>13240721</v>
       </c>
-      <c r="O6" t="inlineStr">
+      <c r="Z6" t="inlineStr">
         <is>
           <t>Optimize HC</t>
         </is>
       </c>
-      <c r="P6" t="n">
+      <c r="AA6" t="n">
         <v>46.7</v>
       </c>
-      <c r="Q6" t="n">
+      <c r="AB6" t="n">
         <v>-0.08400000000000001</v>
       </c>
-      <c r="S6" t="n">
+      <c r="AD6" t="n">
         <v>17780</v>
       </c>
-      <c r="T6" t="n">
+      <c r="AE6" t="n">
         <v>1765233</v>
       </c>
-      <c r="U6" t="n">
+      <c r="AF6" t="n">
         <v>502167251</v>
       </c>
-      <c r="V6" t="n">
+      <c r="AG6" t="n">
         <v>39227</v>
       </c>
-      <c r="W6" t="n">
-        <v>10</v>
-      </c>
-      <c r="X6" t="n">
+      <c r="AH6" t="n">
+        <v>10</v>
+      </c>
+      <c r="AI6" t="n">
         <v>194.28</v>
       </c>
-      <c r="Y6" t="inlineStr">
+      <c r="AJ6" t="inlineStr">
         <is>
           <t>Plateaued</t>
         </is>
       </c>
-      <c r="Z6" t="n">
-        <v>10</v>
-      </c>
-      <c r="AA6" t="n">
+      <c r="AK6" t="n">
+        <v>10</v>
+      </c>
+      <c r="AL6" t="n">
         <v>29</v>
       </c>
-      <c r="AB6" t="n">
+      <c r="AM6" t="n">
         <v>20</v>
       </c>
-      <c r="AC6" t="inlineStr">
+      <c r="AN6" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -1058,83 +1154,89 @@
         <v>78</v>
       </c>
       <c r="E7" t="n">
+        <v>73</v>
+      </c>
+      <c r="I7" t="n">
         <v>131</v>
       </c>
-      <c r="F7" t="n">
+      <c r="J7" t="n">
+        <v>43</v>
+      </c>
+      <c r="K7" t="n">
         <v>53</v>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="L7" t="inlineStr">
         <is>
           <t>Optimize</t>
         </is>
       </c>
-      <c r="H7" t="n">
+      <c r="S7" t="n">
         <v>73</v>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="T7" t="inlineStr">
         <is>
           <t>07: 66-80</t>
         </is>
       </c>
-      <c r="J7" t="n">
+      <c r="U7" t="n">
         <v>80</v>
       </c>
-      <c r="K7" t="n">
+      <c r="V7" t="n">
         <v>0.3</v>
       </c>
-      <c r="L7" t="n">
+      <c r="W7" t="n">
         <v>43</v>
       </c>
-      <c r="M7" t="n">
+      <c r="X7" t="n">
         <v>5669</v>
       </c>
-      <c r="N7" t="n">
+      <c r="Y7" t="n">
         <v>9407836</v>
       </c>
-      <c r="O7" t="inlineStr">
+      <c r="Z7" t="inlineStr">
         <is>
           <t>Optimize HC</t>
         </is>
       </c>
-      <c r="P7" t="n">
+      <c r="AA7" t="n">
         <v>50</v>
       </c>
-      <c r="Q7" t="n">
+      <c r="AB7" t="n">
         <v>0.005</v>
       </c>
-      <c r="S7" t="n">
+      <c r="AD7" t="n">
         <v>3930</v>
       </c>
-      <c r="T7" t="n">
+      <c r="AE7" t="n">
         <v>10886</v>
       </c>
-      <c r="U7" t="n">
+      <c r="AF7" t="n">
         <v>6745421</v>
       </c>
-      <c r="V7" t="n">
+      <c r="AG7" t="n">
         <v>149</v>
       </c>
-      <c r="W7" t="n">
+      <c r="AH7" t="n">
         <v>65</v>
       </c>
-      <c r="X7" t="n">
+      <c r="AI7" t="n">
         <v>44.3</v>
       </c>
-      <c r="Y7" t="inlineStr">
+      <c r="AJ7" t="inlineStr">
         <is>
           <t>Growing</t>
         </is>
       </c>
-      <c r="Z7" t="n">
-        <v>10</v>
-      </c>
-      <c r="AA7" t="n">
+      <c r="AK7" t="n">
+        <v>10</v>
+      </c>
+      <c r="AL7" t="n">
         <v>17</v>
       </c>
-      <c r="AB7" t="n">
+      <c r="AM7" t="n">
         <v>2</v>
       </c>
-      <c r="AC7" t="inlineStr">
+      <c r="AN7" t="inlineStr">
         <is>
           <t>Declining</t>
         </is>
@@ -1160,83 +1262,89 @@
         <v>140</v>
       </c>
       <c r="E8" t="n">
+        <v>15</v>
+      </c>
+      <c r="I8" t="n">
         <v>172</v>
       </c>
-      <c r="F8" t="n">
+      <c r="J8" t="n">
+        <v>12</v>
+      </c>
+      <c r="K8" t="n">
         <v>32</v>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="L8" t="inlineStr">
         <is>
           <t>Optimize</t>
         </is>
       </c>
-      <c r="H8" t="n">
+      <c r="S8" t="n">
         <v>15</v>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="T8" t="inlineStr">
         <is>
           <t>02: 11-20</t>
         </is>
       </c>
-      <c r="J8" t="n">
+      <c r="U8" t="n">
         <v>20</v>
       </c>
-      <c r="K8" t="n">
+      <c r="V8" t="n">
         <v>0.3</v>
       </c>
-      <c r="L8" t="n">
+      <c r="W8" t="n">
         <v>12</v>
       </c>
-      <c r="M8" t="n">
+      <c r="X8" t="n">
         <v>2097</v>
       </c>
-      <c r="N8" t="n">
+      <c r="Y8" t="n">
         <v>8301713</v>
       </c>
-      <c r="O8" t="inlineStr">
+      <c r="Z8" t="inlineStr">
         <is>
           <t>Optimize HC</t>
         </is>
       </c>
-      <c r="P8" t="n">
+      <c r="AA8" t="n">
         <v>49.9</v>
       </c>
-      <c r="Q8" t="n">
+      <c r="AB8" t="n">
         <v>-0.014</v>
       </c>
-      <c r="S8" t="n">
+      <c r="AD8" t="n">
         <v>516</v>
       </c>
-      <c r="T8" t="n">
+      <c r="AE8" t="n">
         <v>1879</v>
       </c>
-      <c r="U8" t="n">
+      <c r="AF8" t="n">
         <v>428831</v>
       </c>
-      <c r="V8" t="n">
+      <c r="AG8" t="n">
         <v>125</v>
       </c>
-      <c r="W8" t="n">
+      <c r="AH8" t="n">
         <v>20</v>
       </c>
-      <c r="X8" t="n">
+      <c r="AI8" t="n">
         <v>7.2</v>
       </c>
-      <c r="Y8" t="inlineStr">
+      <c r="AJ8" t="inlineStr">
         <is>
           <t>Growing</t>
         </is>
       </c>
-      <c r="Z8" t="n">
-        <v>10</v>
-      </c>
-      <c r="AA8" t="n">
+      <c r="AK8" t="n">
+        <v>10</v>
+      </c>
+      <c r="AL8" t="n">
         <v>11</v>
       </c>
-      <c r="AB8" t="n">
+      <c r="AM8" t="n">
         <v>5</v>
       </c>
-      <c r="AC8" t="inlineStr">
+      <c r="AN8" t="inlineStr">
         <is>
           <t>Declining</t>
         </is>
@@ -1262,48 +1370,54 @@
         <v>114</v>
       </c>
       <c r="E9" t="n">
+        <v>5</v>
+      </c>
+      <c r="I9" t="n">
         <v>92</v>
       </c>
-      <c r="F9" t="n">
+      <c r="J9" t="n">
+        <v>6</v>
+      </c>
+      <c r="K9" t="n">
         <v>-22</v>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="L9" t="inlineStr">
         <is>
           <t>Hire</t>
         </is>
       </c>
-      <c r="H9" t="n">
+      <c r="S9" t="n">
         <v>5</v>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="T9" t="inlineStr">
         <is>
           <t>01: 1-10</t>
         </is>
       </c>
-      <c r="J9" t="n">
-        <v>10</v>
-      </c>
-      <c r="K9" t="n">
+      <c r="U9" t="n">
+        <v>10</v>
+      </c>
+      <c r="V9" t="n">
         <v>0.3</v>
       </c>
-      <c r="L9" t="n">
+      <c r="W9" t="n">
         <v>6</v>
       </c>
-      <c r="M9" t="n">
+      <c r="X9" t="n">
         <v>569</v>
       </c>
-      <c r="N9" t="n">
+      <c r="Y9" t="n">
         <v>4126601</v>
       </c>
-      <c r="O9" t="inlineStr">
+      <c r="Z9" t="inlineStr">
         <is>
           <t>Hire</t>
         </is>
       </c>
-      <c r="S9" t="n">
+      <c r="AD9" t="n">
         <v>0</v>
       </c>
-      <c r="V9" t="n">
+      <c r="AG9" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1327,83 +1441,89 @@
         <v>401</v>
       </c>
       <c r="E10" t="n">
+        <v>5</v>
+      </c>
+      <c r="I10" t="n">
         <v>154</v>
       </c>
-      <c r="F10" t="n">
+      <c r="J10" t="n">
+        <v>13</v>
+      </c>
+      <c r="K10" t="n">
         <v>-247</v>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="L10" t="inlineStr">
         <is>
           <t>Hire</t>
         </is>
       </c>
-      <c r="H10" t="n">
+      <c r="S10" t="n">
         <v>5</v>
       </c>
-      <c r="I10" t="inlineStr">
+      <c r="T10" t="inlineStr">
         <is>
           <t>01: 1-10</t>
         </is>
       </c>
-      <c r="J10" t="n">
-        <v>10</v>
-      </c>
-      <c r="K10" t="n">
+      <c r="U10" t="n">
+        <v>10</v>
+      </c>
+      <c r="V10" t="n">
         <v>0.4</v>
       </c>
-      <c r="L10" t="n">
+      <c r="W10" t="n">
         <v>13</v>
       </c>
-      <c r="M10" t="n">
+      <c r="X10" t="n">
         <v>2004</v>
       </c>
-      <c r="N10" t="n">
+      <c r="Y10" t="n">
         <v>4096268</v>
       </c>
-      <c r="O10" t="inlineStr">
+      <c r="Z10" t="inlineStr">
         <is>
           <t>Hire + build books from SBS</t>
         </is>
       </c>
-      <c r="P10" t="n">
+      <c r="AA10" t="n">
         <v>52.8</v>
       </c>
-      <c r="Q10" t="n">
+      <c r="AB10" t="n">
         <v>0.055</v>
       </c>
-      <c r="S10" t="n">
+      <c r="AD10" t="n">
         <v>0</v>
       </c>
-      <c r="T10" t="n">
+      <c r="AE10" t="n">
         <v>1298</v>
       </c>
-      <c r="U10" t="n">
+      <c r="AF10" t="n">
         <v>417037</v>
       </c>
-      <c r="V10" t="n">
+      <c r="AG10" t="n">
         <v>259</v>
       </c>
-      <c r="W10" t="n">
-        <v>10</v>
-      </c>
-      <c r="X10" t="n">
+      <c r="AH10" t="n">
+        <v>10</v>
+      </c>
+      <c r="AI10" t="n">
         <v>10.8</v>
       </c>
-      <c r="Y10" t="inlineStr">
+      <c r="AJ10" t="inlineStr">
         <is>
           <t>Plateaued</t>
         </is>
       </c>
-      <c r="Z10" t="n">
+      <c r="AK10" t="n">
         <v>20</v>
       </c>
-      <c r="AA10" t="n">
+      <c r="AL10" t="n">
         <v>11</v>
       </c>
-      <c r="AB10" t="n">
+      <c r="AM10" t="n">
         <v>8</v>
       </c>
-      <c r="AC10" t="inlineStr">
+      <c r="AN10" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -1429,48 +1549,54 @@
         <v>192</v>
       </c>
       <c r="E11" t="n">
+        <v>5</v>
+      </c>
+      <c r="I11" t="n">
         <v>92</v>
       </c>
-      <c r="F11" t="n">
+      <c r="J11" t="n">
+        <v>10</v>
+      </c>
+      <c r="K11" t="n">
         <v>-100</v>
       </c>
-      <c r="G11" t="inlineStr">
+      <c r="L11" t="inlineStr">
         <is>
           <t>Hire</t>
         </is>
       </c>
-      <c r="H11" t="n">
+      <c r="S11" t="n">
         <v>5</v>
       </c>
-      <c r="I11" t="inlineStr">
+      <c r="T11" t="inlineStr">
         <is>
           <t>01: 1-10</t>
         </is>
       </c>
-      <c r="J11" t="n">
-        <v>10</v>
-      </c>
-      <c r="K11" t="n">
+      <c r="U11" t="n">
+        <v>10</v>
+      </c>
+      <c r="V11" t="n">
         <v>0.3</v>
       </c>
-      <c r="L11" t="n">
-        <v>10</v>
-      </c>
-      <c r="M11" t="n">
+      <c r="W11" t="n">
+        <v>10</v>
+      </c>
+      <c r="X11" t="n">
         <v>960</v>
       </c>
-      <c r="N11" t="n">
+      <c r="Y11" t="n">
         <v>3188432</v>
       </c>
-      <c r="O11" t="inlineStr">
+      <c r="Z11" t="inlineStr">
         <is>
           <t>Hire</t>
         </is>
       </c>
-      <c r="S11" t="n">
+      <c r="AD11" t="n">
         <v>0</v>
       </c>
-      <c r="V11" t="n">
+      <c r="AG11" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1494,48 +1620,54 @@
         <v>101</v>
       </c>
       <c r="E12" t="n">
+        <v>5</v>
+      </c>
+      <c r="I12" t="n">
         <v>88</v>
       </c>
-      <c r="F12" t="n">
+      <c r="J12" t="n">
+        <v>6</v>
+      </c>
+      <c r="K12" t="n">
         <v>-13</v>
       </c>
-      <c r="G12" t="inlineStr">
+      <c r="L12" t="inlineStr">
         <is>
           <t>Hire</t>
         </is>
       </c>
-      <c r="H12" t="n">
+      <c r="S12" t="n">
         <v>5</v>
       </c>
-      <c r="I12" t="inlineStr">
+      <c r="T12" t="inlineStr">
         <is>
           <t>01: 1-10</t>
         </is>
       </c>
-      <c r="J12" t="n">
-        <v>10</v>
-      </c>
-      <c r="K12" t="n">
+      <c r="U12" t="n">
+        <v>10</v>
+      </c>
+      <c r="V12" t="n">
         <v>0.2</v>
       </c>
-      <c r="L12" t="n">
+      <c r="W12" t="n">
         <v>6</v>
       </c>
-      <c r="M12" t="n">
+      <c r="X12" t="n">
         <v>505</v>
       </c>
-      <c r="N12" t="n">
+      <c r="Y12" t="n">
         <v>2748456</v>
       </c>
-      <c r="O12" t="inlineStr">
+      <c r="Z12" t="inlineStr">
         <is>
           <t>Hire</t>
         </is>
       </c>
-      <c r="S12" t="n">
+      <c r="AD12" t="n">
         <v>0</v>
       </c>
-      <c r="V12" t="n">
+      <c r="AG12" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1559,83 +1691,89 @@
         <v>66</v>
       </c>
       <c r="E13" t="n">
+        <v>15</v>
+      </c>
+      <c r="I13" t="n">
         <v>88</v>
       </c>
-      <c r="F13" t="n">
+      <c r="J13" t="n">
+        <v>11</v>
+      </c>
+      <c r="K13" t="n">
         <v>22</v>
       </c>
-      <c r="G13" t="inlineStr">
+      <c r="L13" t="inlineStr">
         <is>
           <t>Optimize</t>
         </is>
       </c>
-      <c r="H13" t="n">
+      <c r="S13" t="n">
         <v>15</v>
       </c>
-      <c r="I13" t="inlineStr">
+      <c r="T13" t="inlineStr">
         <is>
           <t>02: 11-20</t>
         </is>
       </c>
-      <c r="J13" t="n">
+      <c r="U13" t="n">
         <v>20</v>
       </c>
-      <c r="K13" t="n">
+      <c r="V13" t="n">
         <v>0.3</v>
       </c>
-      <c r="L13" t="n">
+      <c r="W13" t="n">
         <v>11</v>
       </c>
-      <c r="M13" t="n">
+      <c r="X13" t="n">
         <v>996</v>
       </c>
-      <c r="N13" t="n">
+      <c r="Y13" t="n">
         <v>2450421</v>
       </c>
-      <c r="O13" t="inlineStr">
+      <c r="Z13" t="inlineStr">
         <is>
           <t>Optimize HC</t>
         </is>
       </c>
-      <c r="P13" t="n">
+      <c r="AA13" t="n">
         <v>49.8</v>
       </c>
-      <c r="Q13" t="n">
+      <c r="AB13" t="n">
         <v>-0.022</v>
       </c>
-      <c r="S13" t="n">
+      <c r="AD13" t="n">
         <v>352</v>
       </c>
-      <c r="T13" t="n">
+      <c r="AE13" t="n">
         <v>599</v>
       </c>
-      <c r="U13" t="n">
+      <c r="AF13" t="n">
         <v>351367</v>
       </c>
-      <c r="V13" t="n">
+      <c r="AG13" t="n">
         <v>39</v>
       </c>
-      <c r="W13" t="n">
+      <c r="AH13" t="n">
         <v>20</v>
       </c>
-      <c r="X13" t="n">
+      <c r="AI13" t="n">
         <v>8.6</v>
       </c>
-      <c r="Y13" t="inlineStr">
+      <c r="AJ13" t="inlineStr">
         <is>
           <t>Growing</t>
         </is>
       </c>
-      <c r="Z13" t="n">
+      <c r="AK13" t="n">
         <v>20</v>
       </c>
-      <c r="AA13" t="n">
+      <c r="AL13" t="n">
         <v>17</v>
       </c>
-      <c r="AB13" t="n">
+      <c r="AM13" t="n">
         <v>6</v>
       </c>
-      <c r="AC13" t="inlineStr">
+      <c r="AN13" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -1661,83 +1799,89 @@
         <v>116</v>
       </c>
       <c r="E14" t="n">
+        <v>5</v>
+      </c>
+      <c r="I14" t="n">
         <v>77</v>
       </c>
-      <c r="F14" t="n">
+      <c r="J14" t="n">
+        <v>8</v>
+      </c>
+      <c r="K14" t="n">
         <v>-39</v>
       </c>
-      <c r="G14" t="inlineStr">
+      <c r="L14" t="inlineStr">
         <is>
           <t>Hire</t>
         </is>
       </c>
-      <c r="H14" t="n">
+      <c r="S14" t="n">
         <v>5</v>
       </c>
-      <c r="I14" t="inlineStr">
+      <c r="T14" t="inlineStr">
         <is>
           <t>01: 1-10</t>
         </is>
       </c>
-      <c r="J14" t="n">
-        <v>10</v>
-      </c>
-      <c r="K14" t="n">
+      <c r="U14" t="n">
+        <v>10</v>
+      </c>
+      <c r="V14" t="n">
         <v>0.3</v>
       </c>
-      <c r="L14" t="n">
+      <c r="W14" t="n">
         <v>8</v>
       </c>
-      <c r="M14" t="n">
+      <c r="X14" t="n">
         <v>582</v>
       </c>
-      <c r="N14" t="n">
+      <c r="Y14" t="n">
         <v>1995476</v>
       </c>
-      <c r="O14" t="inlineStr">
+      <c r="Z14" t="inlineStr">
         <is>
           <t>Hire + build books from SBS</t>
         </is>
       </c>
-      <c r="P14" t="n">
+      <c r="AA14" t="n">
         <v>52.1</v>
       </c>
-      <c r="Q14" t="n">
+      <c r="AB14" t="n">
         <v>0.032</v>
       </c>
-      <c r="S14" t="n">
+      <c r="AD14" t="n">
         <v>0</v>
       </c>
-      <c r="T14" t="n">
+      <c r="AE14" t="n">
         <v>637</v>
       </c>
-      <c r="U14" t="n">
+      <c r="AF14" t="n">
         <v>80994</v>
       </c>
-      <c r="V14" t="n">
+      <c r="AG14" t="n">
         <v>127</v>
       </c>
-      <c r="W14" t="n">
-        <v>10</v>
-      </c>
-      <c r="X14" t="n">
+      <c r="AH14" t="n">
+        <v>10</v>
+      </c>
+      <c r="AI14" t="n">
         <v>0.7</v>
       </c>
-      <c r="Y14" t="inlineStr">
+      <c r="AJ14" t="inlineStr">
         <is>
           <t>Growing</t>
         </is>
       </c>
-      <c r="Z14" t="n">
-        <v>10</v>
-      </c>
-      <c r="AA14" t="n">
+      <c r="AK14" t="n">
+        <v>10</v>
+      </c>
+      <c r="AL14" t="n">
         <v>6</v>
       </c>
-      <c r="AB14" t="n">
+      <c r="AM14" t="n">
         <v>5</v>
       </c>
-      <c r="AC14" t="inlineStr">
+      <c r="AN14" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -1763,48 +1907,54 @@
         <v>403</v>
       </c>
       <c r="E15" t="n">
+        <v>5</v>
+      </c>
+      <c r="I15" t="n">
         <v>122</v>
       </c>
-      <c r="F15" t="n">
+      <c r="J15" t="n">
+        <v>17</v>
+      </c>
+      <c r="K15" t="n">
         <v>-281</v>
       </c>
-      <c r="G15" t="inlineStr">
+      <c r="L15" t="inlineStr">
         <is>
           <t>Hire</t>
         </is>
       </c>
-      <c r="H15" t="n">
+      <c r="S15" t="n">
         <v>5</v>
       </c>
-      <c r="I15" t="inlineStr">
+      <c r="T15" t="inlineStr">
         <is>
           <t>01: 1-10</t>
         </is>
       </c>
-      <c r="J15" t="n">
-        <v>10</v>
-      </c>
-      <c r="K15" t="n">
+      <c r="U15" t="n">
+        <v>10</v>
+      </c>
+      <c r="V15" t="n">
         <v>0.4</v>
       </c>
-      <c r="L15" t="n">
+      <c r="W15" t="n">
         <v>17</v>
       </c>
-      <c r="M15" t="n">
+      <c r="X15" t="n">
         <v>2017</v>
       </c>
-      <c r="N15" t="n">
+      <c r="Y15" t="n">
         <v>1171728</v>
       </c>
-      <c r="O15" t="inlineStr">
+      <c r="Z15" t="inlineStr">
         <is>
           <t>Hire</t>
         </is>
       </c>
-      <c r="S15" t="n">
+      <c r="AD15" t="n">
         <v>0</v>
       </c>
-      <c r="V15" t="n">
+      <c r="AG15" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1828,83 +1978,89 @@
         <v>368</v>
       </c>
       <c r="E16" t="n">
+        <v>5</v>
+      </c>
+      <c r="I16" t="n">
         <v>141</v>
       </c>
-      <c r="F16" t="n">
+      <c r="J16" t="n">
+        <v>13</v>
+      </c>
+      <c r="K16" t="n">
         <v>-227</v>
       </c>
-      <c r="G16" t="inlineStr">
+      <c r="L16" t="inlineStr">
         <is>
           <t>Hire</t>
         </is>
       </c>
-      <c r="H16" t="n">
+      <c r="S16" t="n">
         <v>5</v>
       </c>
-      <c r="I16" t="inlineStr">
+      <c r="T16" t="inlineStr">
         <is>
           <t>01: 1-10</t>
         </is>
       </c>
-      <c r="J16" t="n">
-        <v>10</v>
-      </c>
-      <c r="K16" t="n">
+      <c r="U16" t="n">
+        <v>10</v>
+      </c>
+      <c r="V16" t="n">
         <v>0.3</v>
       </c>
-      <c r="L16" t="n">
+      <c r="W16" t="n">
         <v>13</v>
       </c>
-      <c r="M16" t="n">
+      <c r="X16" t="n">
         <v>1839</v>
       </c>
-      <c r="N16" t="n">
+      <c r="Y16" t="n">
         <v>974670</v>
       </c>
-      <c r="O16" t="inlineStr">
+      <c r="Z16" t="inlineStr">
         <is>
           <t>Hire + build books from SBS</t>
         </is>
       </c>
-      <c r="P16" t="n">
+      <c r="AA16" t="n">
         <v>48.2</v>
       </c>
-      <c r="Q16" t="n">
+      <c r="AB16" t="n">
         <v>-0.048</v>
       </c>
-      <c r="S16" t="n">
+      <c r="AD16" t="n">
         <v>0</v>
       </c>
-      <c r="T16" t="n">
+      <c r="AE16" t="n">
         <v>364298</v>
       </c>
-      <c r="U16" t="n">
+      <c r="AF16" t="n">
         <v>53614691</v>
       </c>
-      <c r="V16" t="n">
+      <c r="AG16" t="n">
         <v>72859</v>
       </c>
-      <c r="W16" t="n">
-        <v>10</v>
-      </c>
-      <c r="X16" t="n">
+      <c r="AH16" t="n">
+        <v>10</v>
+      </c>
+      <c r="AI16" t="n">
         <v>131.6</v>
       </c>
-      <c r="Y16" t="inlineStr">
+      <c r="AJ16" t="inlineStr">
         <is>
           <t>Plateaued</t>
         </is>
       </c>
-      <c r="Z16" t="n">
-        <v>10</v>
-      </c>
-      <c r="AA16" t="n">
+      <c r="AK16" t="n">
+        <v>10</v>
+      </c>
+      <c r="AL16" t="n">
         <v>29</v>
       </c>
-      <c r="AB16" t="n">
+      <c r="AM16" t="n">
         <v>20</v>
       </c>
-      <c r="AC16" t="inlineStr">
+      <c r="AN16" t="inlineStr">
         <is>
           <t>Declining</t>
         </is>
@@ -1930,90 +2086,96 @@
         <v>111</v>
       </c>
       <c r="E17" t="n">
+        <v>5</v>
+      </c>
+      <c r="I17" t="n">
         <v>66</v>
       </c>
-      <c r="F17" t="n">
+      <c r="J17" t="n">
+        <v>8</v>
+      </c>
+      <c r="K17" t="n">
         <v>-45</v>
       </c>
-      <c r="G17" t="inlineStr">
+      <c r="L17" t="inlineStr">
         <is>
           <t>Hire</t>
         </is>
       </c>
-      <c r="H17" t="n">
+      <c r="S17" t="n">
         <v>5</v>
       </c>
-      <c r="I17" t="inlineStr">
+      <c r="T17" t="inlineStr">
         <is>
           <t>01: 1-10</t>
         </is>
       </c>
-      <c r="J17" t="n">
-        <v>10</v>
-      </c>
-      <c r="K17" t="n">
+      <c r="U17" t="n">
+        <v>10</v>
+      </c>
+      <c r="V17" t="n">
         <v>0.2</v>
       </c>
-      <c r="L17" t="n">
+      <c r="W17" t="n">
         <v>8</v>
       </c>
-      <c r="M17" t="n">
+      <c r="X17" t="n">
         <v>556</v>
       </c>
-      <c r="N17" t="n">
+      <c r="Y17" t="n">
         <v>554640</v>
       </c>
-      <c r="O17" t="inlineStr">
+      <c r="Z17" t="inlineStr">
         <is>
           <t>Hire + build books from SBS</t>
         </is>
       </c>
-      <c r="P17" t="n">
+      <c r="AA17" t="n">
         <v>50</v>
       </c>
-      <c r="Q17" t="n">
+      <c r="AB17" t="n">
         <v>-0.006</v>
       </c>
-      <c r="S17" t="n">
+      <c r="AD17" t="n">
         <v>0</v>
       </c>
-      <c r="T17" t="n">
+      <c r="AE17" t="n">
         <v>276061</v>
       </c>
-      <c r="U17" t="n">
+      <c r="AF17" t="n">
         <v>41707962</v>
       </c>
-      <c r="V17" t="n">
+      <c r="AG17" t="n">
         <v>55212</v>
       </c>
-      <c r="W17" t="n">
-        <v>10</v>
-      </c>
-      <c r="X17" t="n">
+      <c r="AH17" t="n">
+        <v>10</v>
+      </c>
+      <c r="AI17" t="n">
         <v>93.8</v>
       </c>
-      <c r="Y17" t="inlineStr">
+      <c r="AJ17" t="inlineStr">
         <is>
           <t>Growing</t>
         </is>
       </c>
-      <c r="Z17" t="n">
-        <v>10</v>
-      </c>
-      <c r="AA17" t="n">
+      <c r="AK17" t="n">
+        <v>10</v>
+      </c>
+      <c r="AL17" t="n">
         <v>20</v>
       </c>
-      <c r="AB17" t="n">
+      <c r="AM17" t="n">
         <v>20</v>
       </c>
-      <c r="AC17" t="inlineStr">
+      <c r="AN17" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AC17"/>
+  <autoFilter ref="A1:AN17"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Refresh dashboard from Quest prod with PQR and book health data.
Merge sql/16 and sql/17 prod exports into headcount.json and book_health.json; fix Trino trailing semicolons and document Quest prod run steps.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/data/headcount-dashboard.xlsx
+++ b/docs/data/headcount-dashboard.xlsx
@@ -685,24 +685,53 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>549</v>
+        <v>552</v>
       </c>
       <c r="E2" t="n">
         <v>73</v>
       </c>
+      <c r="F2" t="n">
+        <v>220303</v>
+      </c>
+      <c r="G2" t="n">
+        <v>163684984</v>
+      </c>
+      <c r="H2" t="n">
+        <v>16.9</v>
+      </c>
       <c r="I2" t="n">
-        <v>735</v>
+        <v>743</v>
       </c>
       <c r="J2" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="K2" t="n">
-        <v>186</v>
+        <v>191</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
           <t>Optimize</t>
         </is>
+      </c>
+      <c r="M2" t="n">
+        <v>421</v>
+      </c>
+      <c r="N2" t="n">
+        <v>369</v>
+      </c>
+      <c r="O2" t="n">
+        <v>8322</v>
+      </c>
+      <c r="P2" t="n">
+        <v>114</v>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>Split-hire 114 new heads (8322 PCIDs pooled)</t>
+        </is>
+      </c>
+      <c r="R2" t="b">
+        <v>1</v>
       </c>
       <c r="S2" t="n">
         <v>73</v>
@@ -716,16 +745,16 @@
         <v>80</v>
       </c>
       <c r="V2" t="n">
-        <v>0.188</v>
+        <v>0.2</v>
       </c>
       <c r="W2" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="X2" t="n">
-        <v>40049</v>
+        <v>40299</v>
       </c>
       <c r="Y2" t="n">
-        <v>191378836</v>
+        <v>191377838</v>
       </c>
       <c r="Z2" t="inlineStr">
         <is>
@@ -739,13 +768,13 @@
         <v>-0.076</v>
       </c>
       <c r="AD2" t="n">
-        <v>13230</v>
+        <v>14117</v>
       </c>
       <c r="AE2" t="n">
-        <v>103681</v>
+        <v>103686</v>
       </c>
       <c r="AF2" t="n">
-        <v>160679658</v>
+        <v>160675164</v>
       </c>
       <c r="AG2" t="n">
         <v>1420</v>
@@ -754,7 +783,7 @@
         <v>100</v>
       </c>
       <c r="AI2" t="n">
-        <v>61.96</v>
+        <v>62</v>
       </c>
       <c r="AJ2" t="inlineStr">
         <is>
@@ -793,24 +822,53 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>1296</v>
+        <v>1306</v>
       </c>
       <c r="E3" t="n">
         <v>5</v>
       </c>
+      <c r="F3" t="n">
+        <v>107286</v>
+      </c>
+      <c r="G3" t="n">
+        <v>97522635</v>
+      </c>
+      <c r="H3" t="n">
+        <v>25.2</v>
+      </c>
       <c r="I3" t="n">
-        <v>906</v>
+        <v>909</v>
       </c>
       <c r="J3" t="n">
         <v>7</v>
       </c>
       <c r="K3" t="n">
-        <v>-390</v>
+        <v>-397</v>
       </c>
       <c r="L3" t="inlineStr">
         <is>
           <t>Hire</t>
         </is>
+      </c>
+      <c r="M3" t="n">
+        <v>346</v>
+      </c>
+      <c r="N3" t="n">
+        <v>216</v>
+      </c>
+      <c r="O3" t="n">
+        <v>2367</v>
+      </c>
+      <c r="P3" t="n">
+        <v>473</v>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>Split-hire 473 new heads (2367 PCIDs pooled)</t>
+        </is>
+      </c>
+      <c r="R3" t="b">
+        <v>1</v>
       </c>
       <c r="S3" t="n">
         <v>5</v>
@@ -830,21 +888,58 @@
         <v>7</v>
       </c>
       <c r="X3" t="n">
-        <v>6482</v>
+        <v>6531</v>
       </c>
       <c r="Y3" t="n">
-        <v>122120633</v>
+        <v>122120636</v>
       </c>
       <c r="Z3" t="inlineStr">
         <is>
-          <t>Hire</t>
-        </is>
+          <t>Hire + build books from SBS</t>
+        </is>
+      </c>
+      <c r="AA3" t="n">
+        <v>51.6</v>
+      </c>
+      <c r="AB3" t="n">
+        <v>0.021</v>
       </c>
       <c r="AD3" t="n">
         <v>0</v>
       </c>
+      <c r="AE3" t="n">
+        <v>23586</v>
+      </c>
+      <c r="AF3" t="n">
+        <v>9633069</v>
+      </c>
       <c r="AG3" t="n">
-        <v>0</v>
+        <v>4717</v>
+      </c>
+      <c r="AH3" t="n">
+        <v>20</v>
+      </c>
+      <c r="AI3" t="n">
+        <v>4.98</v>
+      </c>
+      <c r="AJ3" t="inlineStr">
+        <is>
+          <t>Growing</t>
+        </is>
+      </c>
+      <c r="AK3" t="n">
+        <v>10</v>
+      </c>
+      <c r="AL3" t="n">
+        <v>16</v>
+      </c>
+      <c r="AM3" t="n">
+        <v>9</v>
+      </c>
+      <c r="AN3" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
       </c>
     </row>
     <row r="4">
@@ -864,24 +959,53 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="E4" t="n">
         <v>25</v>
       </c>
+      <c r="F4" t="n">
+        <v>89347</v>
+      </c>
+      <c r="G4" t="n">
+        <v>70583838</v>
+      </c>
+      <c r="H4" t="n">
+        <v>19.9</v>
+      </c>
       <c r="I4" t="n">
-        <v>785</v>
+        <v>790</v>
       </c>
       <c r="J4" t="n">
         <v>15</v>
       </c>
       <c r="K4" t="n">
-        <v>305</v>
+        <v>308</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
           <t>Optimize</t>
         </is>
+      </c>
+      <c r="M4" t="n">
+        <v>328</v>
+      </c>
+      <c r="N4" t="n">
+        <v>600</v>
+      </c>
+      <c r="O4" t="n">
+        <v>701</v>
+      </c>
+      <c r="P4" t="n">
+        <v>28</v>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>Split-hire 28 new heads (701 PCIDs pooled)</t>
+        </is>
+      </c>
+      <c r="R4" t="b">
+        <v>1</v>
       </c>
       <c r="S4" t="n">
         <v>25</v>
@@ -901,21 +1025,58 @@
         <v>15</v>
       </c>
       <c r="X4" t="n">
-        <v>12000</v>
+        <v>12048</v>
       </c>
       <c r="Y4" t="n">
-        <v>84612173</v>
+        <v>84612177</v>
       </c>
       <c r="Z4" t="inlineStr">
         <is>
           <t>Optimize HC</t>
         </is>
       </c>
+      <c r="AA4" t="n">
+        <v>48.3</v>
+      </c>
+      <c r="AB4" t="n">
+        <v>-0.049</v>
+      </c>
       <c r="AD4" t="n">
-        <v>7850</v>
+        <v>7900</v>
+      </c>
+      <c r="AE4" t="n">
+        <v>14873</v>
+      </c>
+      <c r="AF4" t="n">
+        <v>11663037</v>
       </c>
       <c r="AG4" t="n">
-        <v>0</v>
+        <v>594</v>
+      </c>
+      <c r="AH4" t="n">
+        <v>30</v>
+      </c>
+      <c r="AI4" t="n">
+        <v>14.72</v>
+      </c>
+      <c r="AJ4" t="inlineStr">
+        <is>
+          <t>Growing</t>
+        </is>
+      </c>
+      <c r="AK4" t="n">
+        <v>10</v>
+      </c>
+      <c r="AL4" t="n">
+        <v>15</v>
+      </c>
+      <c r="AM4" t="n">
+        <v>4</v>
+      </c>
+      <c r="AN4" t="inlineStr">
+        <is>
+          <t>Declining</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -935,24 +1096,53 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>1313</v>
+        <v>1325</v>
       </c>
       <c r="E5" t="n">
         <v>5</v>
       </c>
+      <c r="F5" t="n">
+        <v>117541</v>
+      </c>
+      <c r="G5" t="n">
+        <v>18924123</v>
+      </c>
+      <c r="H5" t="n">
+        <v>17.8</v>
+      </c>
       <c r="I5" t="n">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="J5" t="n">
         <v>41</v>
       </c>
       <c r="K5" t="n">
-        <v>-1153</v>
+        <v>-1164</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
           <t>Hire</t>
         </is>
+      </c>
+      <c r="M5" t="n">
+        <v>68</v>
+      </c>
+      <c r="N5" t="n">
+        <v>11</v>
+      </c>
+      <c r="O5" t="n">
+        <v>5276</v>
+      </c>
+      <c r="P5" t="n">
+        <v>1055</v>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>Split-hire 1055 new heads (5276 PCIDs pooled)</t>
+        </is>
+      </c>
+      <c r="R5" t="b">
+        <v>1</v>
       </c>
       <c r="S5" t="n">
         <v>5</v>
@@ -972,10 +1162,10 @@
         <v>41</v>
       </c>
       <c r="X5" t="n">
-        <v>6564</v>
+        <v>6627</v>
       </c>
       <c r="Y5" t="n">
-        <v>22290790</v>
+        <v>22290791</v>
       </c>
       <c r="Z5" t="inlineStr">
         <is>
@@ -992,10 +1182,10 @@
         <v>0</v>
       </c>
       <c r="AE5" t="n">
-        <v>17406</v>
+        <v>17408</v>
       </c>
       <c r="AF5" t="n">
-        <v>17062549</v>
+        <v>17062163</v>
       </c>
       <c r="AG5" t="n">
         <v>3481</v>
@@ -1043,24 +1233,53 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="E6" t="n">
         <v>45</v>
       </c>
+      <c r="F6" t="n">
+        <v>20777</v>
+      </c>
+      <c r="G6" t="n">
+        <v>10720937</v>
+      </c>
+      <c r="H6" t="n">
+        <v>23.5</v>
+      </c>
       <c r="I6" t="n">
-        <v>508</v>
+        <v>516</v>
       </c>
       <c r="J6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="K6" t="n">
-        <v>390</v>
+        <v>394</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
           <t>Optimize</t>
         </is>
+      </c>
+      <c r="M6" t="n">
+        <v>100</v>
+      </c>
+      <c r="N6" t="n">
+        <v>278</v>
+      </c>
+      <c r="O6" t="n">
+        <v>61</v>
+      </c>
+      <c r="P6" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>Split-hire 1 new head (61 PCIDs pooled)</t>
+        </is>
+      </c>
+      <c r="R6" t="b">
+        <v>1</v>
       </c>
       <c r="S6" t="n">
         <v>45</v>
@@ -1077,13 +1296,13 @@
         <v>0.2</v>
       </c>
       <c r="W6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X6" t="n">
-        <v>5300</v>
+        <v>5479</v>
       </c>
       <c r="Y6" t="n">
-        <v>13240721</v>
+        <v>13240723</v>
       </c>
       <c r="Z6" t="inlineStr">
         <is>
@@ -1097,22 +1316,22 @@
         <v>-0.08400000000000001</v>
       </c>
       <c r="AD6" t="n">
-        <v>17780</v>
+        <v>17544</v>
       </c>
       <c r="AE6" t="n">
-        <v>1765233</v>
+        <v>1765314</v>
       </c>
       <c r="AF6" t="n">
-        <v>502167251</v>
+        <v>502172154</v>
       </c>
       <c r="AG6" t="n">
-        <v>39227</v>
+        <v>39229</v>
       </c>
       <c r="AH6" t="n">
         <v>10</v>
       </c>
       <c r="AI6" t="n">
-        <v>194.28</v>
+        <v>192.03</v>
       </c>
       <c r="AJ6" t="inlineStr">
         <is>
@@ -1130,7 +1349,7 @@
       </c>
       <c r="AN6" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>Declining</t>
         </is>
       </c>
     </row>
@@ -1151,24 +1370,53 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="E7" t="n">
         <v>73</v>
       </c>
+      <c r="F7" t="n">
+        <v>58766</v>
+      </c>
+      <c r="G7" t="n">
+        <v>7757099</v>
+      </c>
+      <c r="H7" t="n">
+        <v>21.3</v>
+      </c>
       <c r="I7" t="n">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="J7" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="K7" t="n">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="L7" t="inlineStr">
         <is>
           <t>Optimize</t>
         </is>
+      </c>
+      <c r="M7" t="n">
+        <v>54</v>
+      </c>
+      <c r="N7" t="n">
+        <v>57</v>
+      </c>
+      <c r="O7" t="n">
+        <v>539</v>
+      </c>
+      <c r="P7" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>Split-hire 7 new heads (539 PCIDs pooled)</t>
+        </is>
+      </c>
+      <c r="R7" t="b">
+        <v>1</v>
       </c>
       <c r="S7" t="n">
         <v>73</v>
@@ -1185,10 +1433,10 @@
         <v>0.3</v>
       </c>
       <c r="W7" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="X7" t="n">
-        <v>5669</v>
+        <v>5850</v>
       </c>
       <c r="Y7" t="n">
         <v>9407836</v>
@@ -1205,13 +1453,13 @@
         <v>0.005</v>
       </c>
       <c r="AD7" t="n">
-        <v>3930</v>
+        <v>3828</v>
       </c>
       <c r="AE7" t="n">
-        <v>10886</v>
+        <v>10887</v>
       </c>
       <c r="AF7" t="n">
-        <v>6745421</v>
+        <v>6745632</v>
       </c>
       <c r="AG7" t="n">
         <v>149</v>
@@ -1259,11 +1507,20 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="E8" t="n">
         <v>15</v>
       </c>
+      <c r="F8" t="n">
+        <v>38576</v>
+      </c>
+      <c r="G8" t="n">
+        <v>6635068</v>
+      </c>
+      <c r="H8" t="n">
+        <v>25.1</v>
+      </c>
       <c r="I8" t="n">
         <v>172</v>
       </c>
@@ -1271,12 +1528,32 @@
         <v>12</v>
       </c>
       <c r="K8" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="L8" t="inlineStr">
         <is>
           <t>Optimize</t>
         </is>
+      </c>
+      <c r="M8" t="n">
+        <v>57</v>
+      </c>
+      <c r="N8" t="n">
+        <v>81</v>
+      </c>
+      <c r="O8" t="n">
+        <v>368</v>
+      </c>
+      <c r="P8" t="n">
+        <v>24</v>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>Split-hire 24 new heads (368 PCIDs pooled)</t>
+        </is>
+      </c>
+      <c r="R8" t="b">
+        <v>1</v>
       </c>
       <c r="S8" t="n">
         <v>15</v>
@@ -1296,7 +1573,7 @@
         <v>12</v>
       </c>
       <c r="X8" t="n">
-        <v>2097</v>
+        <v>2124</v>
       </c>
       <c r="Y8" t="n">
         <v>8301713</v>
@@ -1316,7 +1593,7 @@
         <v>516</v>
       </c>
       <c r="AE8" t="n">
-        <v>1879</v>
+        <v>1880</v>
       </c>
       <c r="AF8" t="n">
         <v>428831</v>
@@ -1372,6 +1649,15 @@
       <c r="E9" t="n">
         <v>5</v>
       </c>
+      <c r="F9" t="n">
+        <v>34763</v>
+      </c>
+      <c r="G9" t="n">
+        <v>3198151</v>
+      </c>
+      <c r="H9" t="n">
+        <v>29</v>
+      </c>
       <c r="I9" t="n">
         <v>92</v>
       </c>
@@ -1386,6 +1672,26 @@
           <t>Hire</t>
         </is>
       </c>
+      <c r="M9" t="n">
+        <v>26</v>
+      </c>
+      <c r="N9" t="n">
+        <v>12</v>
+      </c>
+      <c r="O9" t="n">
+        <v>169</v>
+      </c>
+      <c r="P9" t="n">
+        <v>33</v>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>Split-hire 33 new heads (169 PCIDs pooled)</t>
+        </is>
+      </c>
+      <c r="R9" t="b">
+        <v>1</v>
+      </c>
       <c r="S9" t="n">
         <v>5</v>
       </c>
@@ -1404,21 +1710,58 @@
         <v>6</v>
       </c>
       <c r="X9" t="n">
-        <v>569</v>
+        <v>570</v>
       </c>
       <c r="Y9" t="n">
         <v>4126601</v>
       </c>
       <c r="Z9" t="inlineStr">
         <is>
-          <t>Hire</t>
-        </is>
+          <t>Hire + build books from SBS</t>
+        </is>
+      </c>
+      <c r="AA9" t="n">
+        <v>52.4</v>
+      </c>
+      <c r="AB9" t="n">
+        <v>0.038</v>
       </c>
       <c r="AD9" t="n">
         <v>0</v>
       </c>
+      <c r="AE9" t="n">
+        <v>2306</v>
+      </c>
+      <c r="AF9" t="n">
+        <v>357161</v>
+      </c>
       <c r="AG9" t="n">
-        <v>0</v>
+        <v>461</v>
+      </c>
+      <c r="AH9" t="n">
+        <v>10</v>
+      </c>
+      <c r="AI9" t="n">
+        <v>6</v>
+      </c>
+      <c r="AJ9" t="inlineStr">
+        <is>
+          <t>Growing</t>
+        </is>
+      </c>
+      <c r="AK9" t="n">
+        <v>10</v>
+      </c>
+      <c r="AL9" t="n">
+        <v>18</v>
+      </c>
+      <c r="AM9" t="n">
+        <v>17</v>
+      </c>
+      <c r="AN9" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
       </c>
     </row>
     <row r="10">
@@ -1438,24 +1781,53 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>401</v>
+        <v>408</v>
       </c>
       <c r="E10" t="n">
         <v>5</v>
       </c>
+      <c r="F10" t="n">
+        <v>22239</v>
+      </c>
+      <c r="G10" t="n">
+        <v>3446995</v>
+      </c>
+      <c r="H10" t="n">
+        <v>18.8</v>
+      </c>
       <c r="I10" t="n">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="J10" t="n">
         <v>13</v>
       </c>
       <c r="K10" t="n">
-        <v>-247</v>
+        <v>-253</v>
       </c>
       <c r="L10" t="inlineStr">
         <is>
           <t>Hire</t>
         </is>
+      </c>
+      <c r="M10" t="n">
+        <v>36</v>
+      </c>
+      <c r="N10" t="n">
+        <v>21</v>
+      </c>
+      <c r="O10" t="n">
+        <v>652</v>
+      </c>
+      <c r="P10" t="n">
+        <v>130</v>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>Split-hire 130 new heads (652 PCIDs pooled)</t>
+        </is>
+      </c>
+      <c r="R10" t="b">
+        <v>1</v>
       </c>
       <c r="S10" t="n">
         <v>5</v>
@@ -1475,7 +1847,7 @@
         <v>13</v>
       </c>
       <c r="X10" t="n">
-        <v>2004</v>
+        <v>2038</v>
       </c>
       <c r="Y10" t="n">
         <v>4096268</v>
@@ -1546,24 +1918,53 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="E11" t="n">
         <v>5</v>
       </c>
+      <c r="F11" t="n">
+        <v>27785</v>
+      </c>
+      <c r="G11" t="n">
+        <v>2556255</v>
+      </c>
+      <c r="H11" t="n">
+        <v>24.7</v>
+      </c>
       <c r="I11" t="n">
         <v>92</v>
       </c>
       <c r="J11" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="K11" t="n">
-        <v>-100</v>
+        <v>-101</v>
       </c>
       <c r="L11" t="inlineStr">
         <is>
           <t>Hire</t>
         </is>
+      </c>
+      <c r="M11" t="n">
+        <v>31</v>
+      </c>
+      <c r="N11" t="n">
+        <v>14</v>
+      </c>
+      <c r="O11" t="n">
+        <v>417</v>
+      </c>
+      <c r="P11" t="n">
+        <v>83</v>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>Split-hire 83 new heads (417 PCIDs pooled)</t>
+        </is>
+      </c>
+      <c r="R11" t="b">
+        <v>1</v>
       </c>
       <c r="S11" t="n">
         <v>5</v>
@@ -1580,24 +1981,61 @@
         <v>0.3</v>
       </c>
       <c r="W11" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X11" t="n">
-        <v>960</v>
+        <v>964</v>
       </c>
       <c r="Y11" t="n">
         <v>3188432</v>
       </c>
       <c r="Z11" t="inlineStr">
         <is>
-          <t>Hire</t>
-        </is>
+          <t>Hire + build books from SBS</t>
+        </is>
+      </c>
+      <c r="AA11" t="n">
+        <v>51.3</v>
+      </c>
+      <c r="AB11" t="n">
+        <v>0.016</v>
       </c>
       <c r="AD11" t="n">
         <v>0</v>
       </c>
+      <c r="AE11" t="n">
+        <v>1610</v>
+      </c>
+      <c r="AF11" t="n">
+        <v>719245</v>
+      </c>
       <c r="AG11" t="n">
-        <v>0</v>
+        <v>322</v>
+      </c>
+      <c r="AH11" t="n">
+        <v>30</v>
+      </c>
+      <c r="AI11" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="AJ11" t="inlineStr">
+        <is>
+          <t>Growing</t>
+        </is>
+      </c>
+      <c r="AK11" t="n">
+        <v>10</v>
+      </c>
+      <c r="AL11" t="n">
+        <v>24</v>
+      </c>
+      <c r="AM11" t="n">
+        <v>7</v>
+      </c>
+      <c r="AN11" t="inlineStr">
+        <is>
+          <t>Declining</t>
+        </is>
       </c>
     </row>
     <row r="12">
@@ -1617,11 +2055,20 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="E12" t="n">
         <v>5</v>
       </c>
+      <c r="F12" t="n">
+        <v>17528</v>
+      </c>
+      <c r="G12" t="n">
+        <v>1542418</v>
+      </c>
+      <c r="H12" t="n">
+        <v>78.2</v>
+      </c>
       <c r="I12" t="n">
         <v>88</v>
       </c>
@@ -1629,12 +2076,32 @@
         <v>6</v>
       </c>
       <c r="K12" t="n">
-        <v>-13</v>
+        <v>-14</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
           <t>Hire</t>
         </is>
+      </c>
+      <c r="M12" t="n">
+        <v>28</v>
+      </c>
+      <c r="N12" t="n">
+        <v>11</v>
+      </c>
+      <c r="O12" t="n">
+        <v>115</v>
+      </c>
+      <c r="P12" t="n">
+        <v>23</v>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>Split-hire 23 new heads (115 PCIDs pooled)</t>
+        </is>
+      </c>
+      <c r="R12" t="b">
+        <v>1</v>
       </c>
       <c r="S12" t="n">
         <v>5</v>
@@ -1654,21 +2121,58 @@
         <v>6</v>
       </c>
       <c r="X12" t="n">
-        <v>505</v>
+        <v>512</v>
       </c>
       <c r="Y12" t="n">
         <v>2748456</v>
       </c>
       <c r="Z12" t="inlineStr">
         <is>
-          <t>Hire</t>
-        </is>
+          <t>Hire + build books from SBS</t>
+        </is>
+      </c>
+      <c r="AA12" t="n">
+        <v>55.4</v>
+      </c>
+      <c r="AB12" t="n">
+        <v>0.08</v>
       </c>
       <c r="AD12" t="n">
         <v>0</v>
       </c>
+      <c r="AE12" t="n">
+        <v>296</v>
+      </c>
+      <c r="AF12" t="n">
+        <v>179218</v>
+      </c>
       <c r="AG12" t="n">
-        <v>0</v>
+        <v>59</v>
+      </c>
+      <c r="AH12" t="n">
+        <v>10</v>
+      </c>
+      <c r="AI12" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="AJ12" t="inlineStr">
+        <is>
+          <t>Growing</t>
+        </is>
+      </c>
+      <c r="AK12" t="n">
+        <v>10</v>
+      </c>
+      <c r="AL12" t="n">
+        <v>30</v>
+      </c>
+      <c r="AM12" t="n">
+        <v>23</v>
+      </c>
+      <c r="AN12" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
       </c>
     </row>
     <row r="13">
@@ -1688,24 +2192,53 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E13" t="n">
         <v>15</v>
       </c>
+      <c r="F13" t="n">
+        <v>22033</v>
+      </c>
+      <c r="G13" t="n">
+        <v>1938921</v>
+      </c>
+      <c r="H13" t="n">
+        <v>26.4</v>
+      </c>
       <c r="I13" t="n">
         <v>88</v>
       </c>
       <c r="J13" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="K13" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
           <t>Optimize</t>
         </is>
+      </c>
+      <c r="M13" t="n">
+        <v>24</v>
+      </c>
+      <c r="N13" t="n">
+        <v>36</v>
+      </c>
+      <c r="O13" t="n">
+        <v>137</v>
+      </c>
+      <c r="P13" t="n">
+        <v>9</v>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>Split-hire 9 new heads (137 PCIDs pooled)</t>
+        </is>
+      </c>
+      <c r="R13" t="b">
+        <v>1</v>
       </c>
       <c r="S13" t="n">
         <v>15</v>
@@ -1722,10 +2255,10 @@
         <v>0.3</v>
       </c>
       <c r="W13" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="X13" t="n">
-        <v>996</v>
+        <v>1008</v>
       </c>
       <c r="Y13" t="n">
         <v>2450421</v>
@@ -1742,7 +2275,7 @@
         <v>-0.022</v>
       </c>
       <c r="AD13" t="n">
-        <v>352</v>
+        <v>264</v>
       </c>
       <c r="AE13" t="n">
         <v>599</v>
@@ -1796,11 +2329,20 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="E14" t="n">
         <v>5</v>
       </c>
+      <c r="F14" t="n">
+        <v>21137</v>
+      </c>
+      <c r="G14" t="n">
+        <v>1627528</v>
+      </c>
+      <c r="H14" t="n">
+        <v>22.6</v>
+      </c>
       <c r="I14" t="n">
         <v>77</v>
       </c>
@@ -1808,12 +2350,32 @@
         <v>8</v>
       </c>
       <c r="K14" t="n">
-        <v>-39</v>
+        <v>-40</v>
       </c>
       <c r="L14" t="inlineStr">
         <is>
           <t>Hire</t>
         </is>
+      </c>
+      <c r="M14" t="n">
+        <v>23</v>
+      </c>
+      <c r="N14" t="n">
+        <v>8</v>
+      </c>
+      <c r="O14" t="n">
+        <v>127</v>
+      </c>
+      <c r="P14" t="n">
+        <v>25</v>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>Split-hire 25 new heads (127 PCIDs pooled)</t>
+        </is>
+      </c>
+      <c r="R14" t="b">
+        <v>1</v>
       </c>
       <c r="S14" t="n">
         <v>5</v>
@@ -1833,7 +2395,7 @@
         <v>8</v>
       </c>
       <c r="X14" t="n">
-        <v>582</v>
+        <v>585</v>
       </c>
       <c r="Y14" t="n">
         <v>1995476</v>
@@ -1853,7 +2415,7 @@
         <v>0</v>
       </c>
       <c r="AE14" t="n">
-        <v>637</v>
+        <v>638</v>
       </c>
       <c r="AF14" t="n">
         <v>80994</v>
@@ -1904,24 +2466,53 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>403</v>
+        <v>459</v>
       </c>
       <c r="E15" t="n">
         <v>5</v>
       </c>
+      <c r="F15" t="n">
+        <v>5214</v>
+      </c>
+      <c r="G15" t="n">
+        <v>641283</v>
+      </c>
+      <c r="H15" t="n">
+        <v>82.7</v>
+      </c>
       <c r="I15" t="n">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="J15" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="K15" t="n">
-        <v>-281</v>
+        <v>-336</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
           <t>Hire</t>
         </is>
+      </c>
+      <c r="M15" t="n">
+        <v>20</v>
+      </c>
+      <c r="N15" t="n">
+        <v>6</v>
+      </c>
+      <c r="O15" t="n">
+        <v>540</v>
+      </c>
+      <c r="P15" t="n">
+        <v>108</v>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>Split-hire 108 new heads (540 PCIDs pooled)</t>
+        </is>
+      </c>
+      <c r="R15" t="b">
+        <v>1</v>
       </c>
       <c r="S15" t="n">
         <v>5</v>
@@ -1938,24 +2529,61 @@
         <v>0.4</v>
       </c>
       <c r="W15" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="X15" t="n">
-        <v>2017</v>
+        <v>2297</v>
       </c>
       <c r="Y15" t="n">
-        <v>1171728</v>
+        <v>1171729</v>
       </c>
       <c r="Z15" t="inlineStr">
         <is>
-          <t>Hire</t>
-        </is>
+          <t>Hire + build books from SBS</t>
+        </is>
+      </c>
+      <c r="AA15" t="n">
+        <v>49.5</v>
+      </c>
+      <c r="AB15" t="n">
+        <v>0.01</v>
       </c>
       <c r="AD15" t="n">
         <v>0</v>
       </c>
+      <c r="AE15" t="n">
+        <v>144336</v>
+      </c>
+      <c r="AF15" t="n">
+        <v>23144861</v>
+      </c>
       <c r="AG15" t="n">
-        <v>0</v>
+        <v>28867</v>
+      </c>
+      <c r="AH15" t="n">
+        <v>10</v>
+      </c>
+      <c r="AI15" t="n">
+        <v>114.3</v>
+      </c>
+      <c r="AJ15" t="inlineStr">
+        <is>
+          <t>Plateaued</t>
+        </is>
+      </c>
+      <c r="AK15" t="n">
+        <v>10</v>
+      </c>
+      <c r="AL15" t="n">
+        <v>30</v>
+      </c>
+      <c r="AM15" t="n">
+        <v>23</v>
+      </c>
+      <c r="AN15" t="inlineStr">
+        <is>
+          <t>Declining</t>
+        </is>
       </c>
     </row>
     <row r="16">
@@ -1975,24 +2603,53 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>368</v>
+        <v>461</v>
       </c>
       <c r="E16" t="n">
         <v>5</v>
       </c>
+      <c r="F16" t="n">
+        <v>4484</v>
+      </c>
+      <c r="G16" t="n">
+        <v>650129</v>
+      </c>
+      <c r="H16" t="n">
+        <v>49.9</v>
+      </c>
       <c r="I16" t="n">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="J16" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="K16" t="n">
-        <v>-227</v>
+        <v>-316</v>
       </c>
       <c r="L16" t="inlineStr">
         <is>
           <t>Hire</t>
         </is>
+      </c>
+      <c r="M16" t="n">
+        <v>16</v>
+      </c>
+      <c r="N16" t="n">
+        <v>15</v>
+      </c>
+      <c r="O16" t="n">
+        <v>547</v>
+      </c>
+      <c r="P16" t="n">
+        <v>109</v>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>Split-hire 109 new heads (547 PCIDs pooled)</t>
+        </is>
+      </c>
+      <c r="R16" t="b">
+        <v>1</v>
       </c>
       <c r="S16" t="n">
         <v>5</v>
@@ -2009,10 +2666,10 @@
         <v>0.3</v>
       </c>
       <c r="W16" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="X16" t="n">
-        <v>1839</v>
+        <v>2304</v>
       </c>
       <c r="Y16" t="n">
         <v>974670</v>
@@ -2032,13 +2689,13 @@
         <v>0</v>
       </c>
       <c r="AE16" t="n">
-        <v>364298</v>
+        <v>364311</v>
       </c>
       <c r="AF16" t="n">
-        <v>53614691</v>
+        <v>53613609</v>
       </c>
       <c r="AG16" t="n">
-        <v>72859</v>
+        <v>72862</v>
       </c>
       <c r="AH16" t="n">
         <v>10</v>
@@ -2083,24 +2740,53 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="E17" t="n">
         <v>5</v>
       </c>
+      <c r="F17" t="n">
+        <v>6469</v>
+      </c>
+      <c r="G17" t="n">
+        <v>426983</v>
+      </c>
+      <c r="H17" t="n">
+        <v>29.9</v>
+      </c>
       <c r="I17" t="n">
         <v>66</v>
       </c>
       <c r="J17" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K17" t="n">
-        <v>-45</v>
+        <v>-47</v>
       </c>
       <c r="L17" t="inlineStr">
         <is>
           <t>Hire</t>
         </is>
+      </c>
+      <c r="M17" t="n">
+        <v>10</v>
+      </c>
+      <c r="N17" t="n">
+        <v>5</v>
+      </c>
+      <c r="O17" t="n">
+        <v>47</v>
+      </c>
+      <c r="P17" t="n">
+        <v>9</v>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>Split-hire 9 new heads (47 PCIDs pooled)</t>
+        </is>
+      </c>
+      <c r="R17" t="b">
+        <v>1</v>
       </c>
       <c r="S17" t="n">
         <v>5</v>
@@ -2117,10 +2803,10 @@
         <v>0.2</v>
       </c>
       <c r="W17" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X17" t="n">
-        <v>556</v>
+        <v>565</v>
       </c>
       <c r="Y17" t="n">
         <v>554640</v>
@@ -2140,13 +2826,13 @@
         <v>0</v>
       </c>
       <c r="AE17" t="n">
-        <v>276061</v>
+        <v>276081</v>
       </c>
       <c r="AF17" t="n">
-        <v>41707962</v>
+        <v>41706619</v>
       </c>
       <c r="AG17" t="n">
-        <v>55212</v>
+        <v>55216</v>
       </c>
       <c r="AH17" t="n">
         <v>10</v>
@@ -2186,7 +2872,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2223,10 +2909,10 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1765233</v>
+        <v>1765314</v>
       </c>
       <c r="D2" t="n">
-        <v>502167251</v>
+        <v>502172154</v>
       </c>
     </row>
     <row r="3">
@@ -2241,10 +2927,10 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>103681</v>
+        <v>103686</v>
       </c>
       <c r="D3" t="n">
-        <v>160679658</v>
+        <v>160675164</v>
       </c>
     </row>
     <row r="4">
@@ -2259,10 +2945,10 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>364298</v>
+        <v>364311</v>
       </c>
       <c r="D4" t="n">
-        <v>53614691</v>
+        <v>53613609</v>
       </c>
     </row>
     <row r="5">
@@ -2277,34 +2963,34 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>276061</v>
+        <v>276081</v>
       </c>
       <c r="D5" t="n">
-        <v>41707962</v>
+        <v>41706619</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>UK</t>
+          <t>DACH</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>17406</v>
+        <v>144336</v>
       </c>
       <c r="D6" t="n">
-        <v>17062549</v>
+        <v>23144861</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>DACH</t>
+          <t>UK</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -2313,16 +2999,16 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>10886</v>
+        <v>17408</v>
       </c>
       <c r="D7" t="n">
-        <v>6745421</v>
+        <v>17062163</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>UK</t>
+          <t>US</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -2331,63 +3017,171 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>1879</v>
+        <v>14873</v>
       </c>
       <c r="D8" t="n">
-        <v>428831</v>
+        <v>11663037</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>DACH</t>
+          <t>US</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>XL</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>1298</v>
+        <v>23586</v>
       </c>
       <c r="D9" t="n">
-        <v>417037</v>
+        <v>9633069</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>BNL</t>
+          <t>DACH</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>M</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>599</v>
+        <v>10887</v>
       </c>
       <c r="D10" t="n">
-        <v>351367</v>
+        <v>6745632</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>1610</v>
+      </c>
+      <c r="D11" t="n">
+        <v>719245</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>1880</v>
+      </c>
+      <c r="D12" t="n">
+        <v>428831</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>DACH</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>1298</v>
+      </c>
+      <c r="D13" t="n">
+        <v>417037</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>XL</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>2306</v>
+      </c>
+      <c r="D14" t="n">
+        <v>357161</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>BNL</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>599</v>
+      </c>
+      <c r="D15" t="n">
+        <v>351367</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>BNL</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>XL</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>296</v>
+      </c>
+      <c r="D16" t="n">
+        <v>179218</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
           <t>FR</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>XL</t>
         </is>
       </c>
-      <c r="C11" t="n">
-        <v>637</v>
-      </c>
-      <c r="D11" t="n">
+      <c r="C17" t="n">
+        <v>638</v>
+      </c>
+      <c r="D17" t="n">
         <v>80994</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add optimal book panel and PQR/PCID methodology to dashboard.
Surfaces data-derived ideal PCID rationale per segment in the lookup UI, expandable methodology, market summaries, and Excel export.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/data/headcount-dashboard.xlsx
+++ b/docs/data/headcount-dashboard.xlsx
@@ -15,11 +15,11 @@
     <sheet name="About" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Markets'!$A$1:$AX$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Markets'!$A$1:$BA$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Rep book'!$A$1:$R$1080</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Book health (flagged reps)'!$A$1:$P$720</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'SBS whitespace'!$A$1:$D$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Market summaries'!$A$1:$I$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Market summaries'!$A$1:$N$9</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AX9"/>
+  <dimension ref="A1:BA9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -481,6 +481,9 @@
     <col width="31" customWidth="1" min="48" max="48"/>
     <col width="29" customWidth="1" min="49" max="49"/>
     <col width="26" customWidth="1" min="50" max="50"/>
+    <col width="36" customWidth="1" min="51" max="51"/>
+    <col width="34" customWidth="1" min="52" max="52"/>
+    <col width="31" customWidth="1" min="53" max="53"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -734,6 +737,21 @@
           <t>Summary — full narrative</t>
         </is>
       </c>
+      <c r="AY1" s="1" t="inlineStr">
+        <is>
+          <t>Optimal book — why (plain English)</t>
+        </is>
+      </c>
+      <c r="AZ1" s="1" t="inlineStr">
+        <is>
+          <t>Optimal book — supporting detail</t>
+        </is>
+      </c>
+      <c r="BA1" s="1" t="inlineStr">
+        <is>
+          <t>Optimal book — full rationale</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -901,12 +919,27 @@
       </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>Book health: 77 reps flagged too big, 1 too little (uneven books across the team). · PQR trend: Revenue is 17.6% above prior-quarter PQR (Hire signal from capacity model). · SBS whitespace: 1,908,879 unassigned accounts in this country × segment (~21,209 buildable books at ideal size). · Split-hire: Model suggests 85 new heads from 7,699 pooled PCIDs — Split-hire 85 new heads (7699 PCIDs pooled) · Market signals: opp pipeline plateaued, coverage ok. · FY26 book build: 46.3% of policy flags positive — room to improve book quality. · Recommended next step: Hire + build books from SBS.</t>
+          <t>Optimal book for this segment is 90 accounts/rep (81-100 band). We pick the largest book-size bucket where median revenue growth stays within 85% of the segment peak (20% in that band) and a bigger book no longer adds growth — that plateau is the data-driven target for headcount math. · Book health: 77 reps flagged too big, 1 too little (uneven books across the team). · PQR trend: Revenue is 17.6% above prior-quarter PQR (Hire signal from capacity model). · SBS whitespace: 1,908,879 unassigned accounts in this country × segment (~21,209 buildable books at ideal size). · Split-hire: Model suggests 85 new heads from 7,699 pooled PCIDs — Split-hire 85 new heads (7699 PCIDs pooled) · Market signals: opp pipeline plateaued, coverage ok. · FY26 book build: 46.3% of policy flags positive — room to improve book quality. · Recommended next step: Hire + build books from SBS.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
         <is>
-          <t>Under headcount by 93 reps (227 current vs 320 ideal). Avg book 127 vs ideal 90 — headcount is short but existing books are already above ideal; prioritize split/redistribution before pure hiring. Book health: 77 reps flagged too big, 1 too little (uneven books across the team). PQR trend: Revenue is 17.6% above prior-quarter PQR (Hire signal from capacity model). SBS whitespace: 1,908,879 unassigned accounts in this country × segment (~21,209 buildable books at ideal size). Split-hire: Model suggests 85 new heads from 7,699 pooled PCIDs — Split-hire 85 new heads (7699 PCIDs pooled) Market signals: opp pipeline plateaued, coverage ok. FY26 book build: 46.3% of policy flags positive — room to improve book quality. Recommended next step: Hire + build books from SBS.</t>
+          <t>Under headcount by 93 reps (227 current vs 320 ideal). Avg book 127 vs ideal 90 — headcount is short but existing books are already above ideal; prioritize split/redistribution before pure hiring. Optimal book for this segment is 90 accounts/rep (81-100 band). We pick the largest book-size bucket where median revenue growth stays within 85% of the segment peak (20% in that band) and a bigger book no longer adds growth — that plateau is the data-driven target for headcount math. Book health: 77 reps flagged too big, 1 too little (uneven books across the team). PQR trend: Revenue is 17.6% above prior-quarter PQR (Hire signal from capacity model). SBS whitespace: 1,908,879 unassigned accounts in this country × segment (~21,209 buildable books at ideal size). Split-hire: Model suggests 85 new heads from 7,699 pooled PCIDs — Split-hire 85 new heads (7699 PCIDs pooled) Market signals: opp pipeline plateaued, coverage ok. FY26 book build: 46.3% of policy flags positive — room to improve book quality. Recommended next step: Hire + build books from SBS.</t>
+        </is>
+      </c>
+      <c r="AY2" t="inlineStr">
+        <is>
+          <t>Optimal book for this segment is 90 accounts/rep (81-100 band). We pick the largest book-size bucket where median revenue growth stays within 85% of the segment peak (20% in that band) and a bigger book no longer adds growth — that plateau is the data-driven target for headcount math.</t>
+        </is>
+      </c>
+      <c r="AZ2" t="inlineStr">
+        <is>
+          <t>Segment avg PQR (prior quarter revenue per rep): $407K — the benchmark for whether a rep's book is revenue-heavy vs peers. · Segment avg PCID: 125 accounts/rep — typical book size today; ideal PCID is the growth-optimal target, not the average. · Current avg book (127) is above ideal — more accounts per rep can dilute coverage and drag growth; peel toward ideal PCID. · Opp pipeline plateaus around 100 accounts/rep — revenue per job peaks near this book size. · Coverage (impact calls/account) peaks near 100 accounts/rep — books larger than this tend to see fewer touches per account. · Too big = PCID or PQR above segment avg plus weak coverage or revenue below PQR; too little = below ideal PCID. Split/peel actions use ideal PCID as the target.</t>
+        </is>
+      </c>
+      <c r="BA2" t="inlineStr">
+        <is>
+          <t>Optimal book for this segment is 90 accounts/rep (81-100 band). We pick the largest book-size bucket where median revenue growth stays within 85% of the segment peak (20% in that band) and a bigger book no longer adds growth — that plateau is the data-driven target for headcount math. Segment avg PQR (prior quarter revenue per rep): $407K — the benchmark for whether a rep's book is revenue-heavy vs peers. Segment avg PCID: 125 accounts/rep — typical book size today; ideal PCID is the growth-optimal target, not the average. Current avg book (127) is above ideal — more accounts per rep can dilute coverage and drag growth; peel toward ideal PCID. Opp pipeline plateaus around 100 accounts/rep — revenue per job peaks near this book size. Coverage (impact calls/account) peaks near 100 accounts/rep — books larger than this tend to see fewer touches per account. Too big = PCID or PQR above segment avg plus weak coverage or revenue below PQR; too little = below ideal PCID. Split/peel actions use ideal PCID as the target.</t>
         </is>
       </c>
     </row>
@@ -1076,12 +1109,27 @@
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>Book health: 81 reps flagged too big, 204 too little (uneven books across the team). · PQR trend: Revenue is 20.5% above prior-quarter PQR (Optimize signal from capacity model). · SBS whitespace: 1,908,879 unassigned accounts in this country × segment (~32,911 buildable books at ideal size). · Book action: Redistribute internally (too big → too little). · Market signals: opp pipeline growing, coverage ok. · FY26 book build: 49.1% of policy flags positive — room to improve book quality. · Recommended next step: Optimize HC.</t>
+          <t>Optimal book for this segment is 58 accounts/rep (51-65 band). We pick the largest book-size bucket where median revenue growth stays within 85% of the segment peak (20% in that band) and a bigger book no longer adds growth — that plateau is the data-driven target for headcount math. · Book health: 81 reps flagged too big, 204 too little (uneven books across the team). · PQR trend: Revenue is 20.5% above prior-quarter PQR (Optimize signal from capacity model). · SBS whitespace: 1,908,879 unassigned accounts in this country × segment (~32,911 buildable books at ideal size). · Book action: Redistribute internally (too big → too little). · Market signals: opp pipeline growing, coverage ok. · FY26 book build: 49.1% of policy flags positive — room to improve book quality. · Recommended next step: Optimize HC.</t>
         </is>
       </c>
       <c r="AX3" t="inlineStr">
         <is>
-          <t>Over headcount by 68 reps (212 current vs 144 ideal). Avg book 39 vs ideal 58 — books are underweight even though we carry more reps than the capacity model needs. Book health: 81 reps flagged too big, 204 too little (uneven books across the team). PQR trend: Revenue is 20.5% above prior-quarter PQR (Optimize signal from capacity model). SBS whitespace: 1,908,879 unassigned accounts in this country × segment (~32,911 buildable books at ideal size). Book action: Redistribute internally (too big → too little). Market signals: opp pipeline growing, coverage ok. FY26 book build: 49.1% of policy flags positive — room to improve book quality. Recommended next step: Optimize HC.</t>
+          <t>Over headcount by 68 reps (212 current vs 144 ideal). Avg book 39 vs ideal 58 — books are underweight even though we carry more reps than the capacity model needs. Optimal book for this segment is 58 accounts/rep (51-65 band). We pick the largest book-size bucket where median revenue growth stays within 85% of the segment peak (20% in that band) and a bigger book no longer adds growth — that plateau is the data-driven target for headcount math. Book health: 81 reps flagged too big, 204 too little (uneven books across the team). PQR trend: Revenue is 20.5% above prior-quarter PQR (Optimize signal from capacity model). SBS whitespace: 1,908,879 unassigned accounts in this country × segment (~32,911 buildable books at ideal size). Book action: Redistribute internally (too big → too little). Market signals: opp pipeline growing, coverage ok. FY26 book build: 49.1% of policy flags positive — room to improve book quality. Recommended next step: Optimize HC.</t>
+        </is>
+      </c>
+      <c r="AY3" t="inlineStr">
+        <is>
+          <t>Optimal book for this segment is 58 accounts/rep (51-65 band). We pick the largest book-size bucket where median revenue growth stays within 85% of the segment peak (20% in that band) and a bigger book no longer adds growth — that plateau is the data-driven target for headcount math.</t>
+        </is>
+      </c>
+      <c r="AZ3" t="inlineStr">
+        <is>
+          <t>Segment avg PQR (prior quarter revenue per rep): $415K — the benchmark for whether a rep's book is revenue-heavy vs peers. · Segment avg PCID: 40 accounts/rep — typical book size today; ideal PCID is the growth-optimal target, not the average. · Current avg book (39) is below ideal — room to grow books toward the growth-optimal size before adding headcount. · Opp pipeline still growing around 50 accounts/rep — revenue per job peaks near this book size. · Coverage (impact calls/account) peaks near 65 accounts/rep — books larger than this tend to see fewer touches per account. · Too big = PCID or PQR above segment avg plus weak coverage or revenue below PQR; too little = below ideal PCID. Split/peel actions use ideal PCID as the target.</t>
+        </is>
+      </c>
+      <c r="BA3" t="inlineStr">
+        <is>
+          <t>Optimal book for this segment is 58 accounts/rep (51-65 band). We pick the largest book-size bucket where median revenue growth stays within 85% of the segment peak (20% in that band) and a bigger book no longer adds growth — that plateau is the data-driven target for headcount math. Segment avg PQR (prior quarter revenue per rep): $415K — the benchmark for whether a rep's book is revenue-heavy vs peers. Segment avg PCID: 40 accounts/rep — typical book size today; ideal PCID is the growth-optimal target, not the average. Current avg book (39) is below ideal — room to grow books toward the growth-optimal size before adding headcount. Opp pipeline still growing around 50 accounts/rep — revenue per job peaks near this book size. Coverage (impact calls/account) peaks near 65 accounts/rep — books larger than this tend to see fewer touches per account. Too big = PCID or PQR above segment avg plus weak coverage or revenue below PQR; too little = below ideal PCID. Split/peel actions use ideal PCID as the target.</t>
         </is>
       </c>
     </row>
@@ -1251,12 +1299,27 @@
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>Book health: 108 reps flagged too big, 57 too little (uneven books across the team). · PQR trend: Revenue is 29.0% above prior-quarter PQR (Hire signal from capacity model). · SBS whitespace: 1,908,879 unassigned accounts in this country × segment (~381,775 buildable books at ideal size). · Split-hire: Model suggests 473 new heads from 2,369 pooled PCIDs — Split-hire 473 new heads (2369 PCIDs pooled) · Market signals: opp pipeline growing, coverage ok. · Recommended next step: Hire + build books from SBS.</t>
+          <t>Optimal book for this segment is 5 accounts/rep (1-10 band). We pick the largest book-size bucket where median revenue growth stays within 85% of the segment peak (23% in that band) and a bigger book no longer adds growth — that plateau is the data-driven target for headcount math. · Book health: 108 reps flagged too big, 57 too little (uneven books across the team). · PQR trend: Revenue is 29.0% above prior-quarter PQR (Hire signal from capacity model). · SBS whitespace: 1,908,879 unassigned accounts in this country × segment (~381,775 buildable books at ideal size). · Split-hire: Model suggests 473 new heads from 2,369 pooled PCIDs — Split-hire 473 new heads (2369 PCIDs pooled) · Market signals: opp pipeline growing, coverage ok. · Recommended next step: Hire + build books from SBS.</t>
         </is>
       </c>
       <c r="AX4" t="inlineStr">
         <is>
-          <t>Under headcount by 520 reps (232 current vs 752 ideal). Avg book 16 vs ideal 5 — headcount is short but existing books are already above ideal; prioritize split/redistribution before pure hiring. Book health: 108 reps flagged too big, 57 too little (uneven books across the team). PQR trend: Revenue is 29.0% above prior-quarter PQR (Hire signal from capacity model). SBS whitespace: 1,908,879 unassigned accounts in this country × segment (~381,775 buildable books at ideal size). Split-hire: Model suggests 473 new heads from 2,369 pooled PCIDs — Split-hire 473 new heads (2369 PCIDs pooled) Market signals: opp pipeline growing, coverage ok. Recommended next step: Hire + build books from SBS.</t>
+          <t>Under headcount by 520 reps (232 current vs 752 ideal). Avg book 16 vs ideal 5 — headcount is short but existing books are already above ideal; prioritize split/redistribution before pure hiring. Optimal book for this segment is 5 accounts/rep (1-10 band). We pick the largest book-size bucket where median revenue growth stays within 85% of the segment peak (23% in that band) and a bigger book no longer adds growth — that plateau is the data-driven target for headcount math. Book health: 108 reps flagged too big, 57 too little (uneven books across the team). PQR trend: Revenue is 29.0% above prior-quarter PQR (Hire signal from capacity model). SBS whitespace: 1,908,879 unassigned accounts in this country × segment (~381,775 buildable books at ideal size). Split-hire: Model suggests 473 new heads from 2,369 pooled PCIDs — Split-hire 473 new heads (2369 PCIDs pooled) Market signals: opp pipeline growing, coverage ok. Recommended next step: Hire + build books from SBS.</t>
+        </is>
+      </c>
+      <c r="AY4" t="inlineStr">
+        <is>
+          <t>Optimal book for this segment is 5 accounts/rep (1-10 band). We pick the largest book-size bucket where median revenue growth stays within 85% of the segment peak (23% in that band) and a bigger book no longer adds growth — that plateau is the data-driven target for headcount math.</t>
+        </is>
+      </c>
+      <c r="AZ4" t="inlineStr">
+        <is>
+          <t>Segment avg PQR (prior quarter revenue per rep): $249K — the benchmark for whether a rep's book is revenue-heavy vs peers. · Segment avg PCID: 16 accounts/rep — typical book size today; ideal PCID is the growth-optimal target, not the average. · Current avg book (16) is above ideal — more accounts per rep can dilute coverage and drag growth; peel toward ideal PCID. · Opp pipeline still growing around 50 accounts/rep — revenue per job peaks near this book size. · Coverage (impact calls/account) peaks near 50 accounts/rep — books larger than this tend to see fewer touches per account. · Too big = PCID or PQR above segment avg plus weak coverage or revenue below PQR; too little = below ideal PCID. Split/peel actions use ideal PCID as the target.</t>
+        </is>
+      </c>
+      <c r="BA4" t="inlineStr">
+        <is>
+          <t>Optimal book for this segment is 5 accounts/rep (1-10 band). We pick the largest book-size bucket where median revenue growth stays within 85% of the segment peak (23% in that band) and a bigger book no longer adds growth — that plateau is the data-driven target for headcount math. Segment avg PQR (prior quarter revenue per rep): $249K — the benchmark for whether a rep's book is revenue-heavy vs peers. Segment avg PCID: 16 accounts/rep — typical book size today; ideal PCID is the growth-optimal target, not the average. Current avg book (16) is above ideal — more accounts per rep can dilute coverage and drag growth; peel toward ideal PCID. Opp pipeline still growing around 50 accounts/rep — revenue per job peaks near this book size. Coverage (impact calls/account) peaks near 50 accounts/rep — books larger than this tend to see fewer touches per account. Too big = PCID or PQR above segment avg plus weak coverage or revenue below PQR; too little = below ideal PCID. Split/peel actions use ideal PCID as the target.</t>
         </is>
       </c>
     </row>
@@ -1426,12 +1489,27 @@
       </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>Book health: 39 reps flagged too big, 3 too little (uneven books across the team). · PQR trend: Revenue is 17.7% above prior-quarter PQR (Hold signal from capacity model). · SBS whitespace: 1,908,879 unassigned accounts in this country × segment (~32,911 buildable books at ideal size). · Split-hire: Model suggests 3 new heads from 199 pooled PCIDs — Split-hire 3 new heads (199 PCIDs pooled) · Market signals: opp pipeline growing, coverage ok. · FY26 book build: 47.4% of policy flags positive — room to improve book quality. · Recommended next step: Improve FY26 book build score.</t>
+          <t>Optimal book for this segment is 58 accounts/rep (51-65 band). We pick the largest book-size bucket where median revenue growth stays within 85% of the segment peak (20% in that band) and a bigger book no longer adds growth — that plateau is the data-driven target for headcount math. · Book health: 39 reps flagged too big, 3 too little (uneven books across the team). · PQR trend: Revenue is 17.7% above prior-quarter PQR (Hold signal from capacity model). · SBS whitespace: 1,908,879 unassigned accounts in this country × segment (~32,911 buildable books at ideal size). · Split-hire: Model suggests 3 new heads from 199 pooled PCIDs — Split-hire 3 new heads (199 PCIDs pooled) · Market signals: opp pipeline growing, coverage ok. · FY26 book build: 47.4% of policy flags positive — room to improve book quality. · Recommended next step: Improve FY26 book build score.</t>
         </is>
       </c>
       <c r="AX5" t="inlineStr">
         <is>
-          <t>Near target headcount (134 current vs 141 ideal, gap -7). Avg book 61 vs ideal 58 — both headcount and book size are close to model. Book health: 39 reps flagged too big, 3 too little (uneven books across the team). PQR trend: Revenue is 17.7% above prior-quarter PQR (Hold signal from capacity model). SBS whitespace: 1,908,879 unassigned accounts in this country × segment (~32,911 buildable books at ideal size). Split-hire: Model suggests 3 new heads from 199 pooled PCIDs — Split-hire 3 new heads (199 PCIDs pooled) Market signals: opp pipeline growing, coverage ok. FY26 book build: 47.4% of policy flags positive — room to improve book quality. Recommended next step: Improve FY26 book build score.</t>
+          <t>Near target headcount (134 current vs 141 ideal, gap -7). Avg book 61 vs ideal 58 — both headcount and book size are close to model. Optimal book for this segment is 58 accounts/rep (51-65 band). We pick the largest book-size bucket where median revenue growth stays within 85% of the segment peak (20% in that band) and a bigger book no longer adds growth — that plateau is the data-driven target for headcount math. Book health: 39 reps flagged too big, 3 too little (uneven books across the team). PQR trend: Revenue is 17.7% above prior-quarter PQR (Hold signal from capacity model). SBS whitespace: 1,908,879 unassigned accounts in this country × segment (~32,911 buildable books at ideal size). Split-hire: Model suggests 3 new heads from 199 pooled PCIDs — Split-hire 3 new heads (199 PCIDs pooled) Market signals: opp pipeline growing, coverage ok. FY26 book build: 47.4% of policy flags positive — room to improve book quality. Recommended next step: Improve FY26 book build score.</t>
+        </is>
+      </c>
+      <c r="AY5" t="inlineStr">
+        <is>
+          <t>Optimal book for this segment is 58 accounts/rep (51-65 band). We pick the largest book-size bucket where median revenue growth stays within 85% of the segment peak (20% in that band) and a bigger book no longer adds growth — that plateau is the data-driven target for headcount math.</t>
+        </is>
+      </c>
+      <c r="AZ5" t="inlineStr">
+        <is>
+          <t>Segment avg PQR (prior quarter revenue per rep): $387K — the benchmark for whether a rep's book is revenue-heavy vs peers. · Segment avg PCID: 61 accounts/rep — typical book size today; ideal PCID is the growth-optimal target, not the average. · Opp pipeline still growing around 65 accounts/rep — revenue per job peaks near this book size. · Coverage (impact calls/account) peaks near 65 accounts/rep — books larger than this tend to see fewer touches per account. · Too big = PCID or PQR above segment avg plus weak coverage or revenue below PQR; too little = below ideal PCID. Split/peel actions use ideal PCID as the target.</t>
+        </is>
+      </c>
+      <c r="BA5" t="inlineStr">
+        <is>
+          <t>Optimal book for this segment is 58 accounts/rep (51-65 band). We pick the largest book-size bucket where median revenue growth stays within 85% of the segment peak (20% in that band) and a bigger book no longer adds growth — that plateau is the data-driven target for headcount math. Segment avg PQR (prior quarter revenue per rep): $387K — the benchmark for whether a rep's book is revenue-heavy vs peers. Segment avg PCID: 61 accounts/rep — typical book size today; ideal PCID is the growth-optimal target, not the average. Opp pipeline still growing around 65 accounts/rep — revenue per job peaks near this book size. Coverage (impact calls/account) peaks near 65 accounts/rep — books larger than this tend to see fewer touches per account. Too big = PCID or PQR above segment avg plus weak coverage or revenue below PQR; too little = below ideal PCID. Split/peel actions use ideal PCID as the target.</t>
         </is>
       </c>
     </row>
@@ -1589,12 +1667,27 @@
       </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>Book health: 69 reps flagged too big, 72 too little (uneven books across the team). · PQR trend: Revenue is 16.2% above prior-quarter PQR (Optimize signal from capacity model). · SBS whitespace: 1,908,879 unassigned accounts in this country × segment (~13,832 buildable books at ideal size). · Split-hire: Model suggests 2 new heads from 306 pooled PCIDs — Split-hire 2 new heads (306 PCIDs pooled) · Market signals: opp pipeline unknown, coverage ok. · FY26 book build: 45.0% of policy flags positive — room to improve book quality. · Recommended next step: Optimize HC.</t>
+          <t>Optimal book for this segment is 138 accounts/rep (126-150 band). We pick the largest book-size bucket where median revenue growth stays within 85% of the segment peak (20% in that band) and a bigger book no longer adds growth — that plateau is the data-driven target for headcount math. · Book health: 69 reps flagged too big, 72 too little (uneven books across the team). · PQR trend: Revenue is 16.2% above prior-quarter PQR (Optimize signal from capacity model). · SBS whitespace: 1,908,879 unassigned accounts in this country × segment (~13,832 buildable books at ideal size). · Split-hire: Model suggests 2 new heads from 306 pooled PCIDs — Split-hire 2 new heads (306 PCIDs pooled) · Market signals: opp pipeline unknown, coverage ok. · FY26 book build: 45.0% of policy flags positive — room to improve book quality. · Recommended next step: Optimize HC.</t>
         </is>
       </c>
       <c r="AX6" t="inlineStr">
         <is>
-          <t>Over headcount by 31 reps (111 current vs 80 ideal). Avg book 99 vs ideal 138 — books are underweight even though we carry more reps than the capacity model needs. Book health: 69 reps flagged too big, 72 too little (uneven books across the team). PQR trend: Revenue is 16.2% above prior-quarter PQR (Optimize signal from capacity model). SBS whitespace: 1,908,879 unassigned accounts in this country × segment (~13,832 buildable books at ideal size). Split-hire: Model suggests 2 new heads from 306 pooled PCIDs — Split-hire 2 new heads (306 PCIDs pooled) Market signals: opp pipeline unknown, coverage ok. FY26 book build: 45.0% of policy flags positive — room to improve book quality. Recommended next step: Optimize HC.</t>
+          <t>Over headcount by 31 reps (111 current vs 80 ideal). Avg book 99 vs ideal 138 — books are underweight even though we carry more reps than the capacity model needs. Optimal book for this segment is 138 accounts/rep (126-150 band). We pick the largest book-size bucket where median revenue growth stays within 85% of the segment peak (20% in that band) and a bigger book no longer adds growth — that plateau is the data-driven target for headcount math. Book health: 69 reps flagged too big, 72 too little (uneven books across the team). PQR trend: Revenue is 16.2% above prior-quarter PQR (Optimize signal from capacity model). SBS whitespace: 1,908,879 unassigned accounts in this country × segment (~13,832 buildable books at ideal size). Split-hire: Model suggests 2 new heads from 306 pooled PCIDs — Split-hire 2 new heads (306 PCIDs pooled) Market signals: opp pipeline unknown, coverage ok. FY26 book build: 45.0% of policy flags positive — room to improve book quality. Recommended next step: Optimize HC.</t>
+        </is>
+      </c>
+      <c r="AY6" t="inlineStr">
+        <is>
+          <t>Optimal book for this segment is 138 accounts/rep (126-150 band). We pick the largest book-size bucket where median revenue growth stays within 85% of the segment peak (20% in that band) and a bigger book no longer adds growth — that plateau is the data-driven target for headcount math.</t>
+        </is>
+      </c>
+      <c r="AZ6" t="inlineStr">
+        <is>
+          <t>Segment avg PQR (prior quarter revenue per rep): $413K — the benchmark for whether a rep's book is revenue-heavy vs peers. · Segment avg PCID: 107 accounts/rep — typical book size today; ideal PCID is the growth-optimal target, not the average. · Current avg book (99) is below ideal — room to grow books toward the growth-optimal size before adding headcount. · Too big = PCID or PQR above segment avg plus weak coverage or revenue below PQR; too little = below ideal PCID. Split/peel actions use ideal PCID as the target.</t>
+        </is>
+      </c>
+      <c r="BA6" t="inlineStr">
+        <is>
+          <t>Optimal book for this segment is 138 accounts/rep (126-150 band). We pick the largest book-size bucket where median revenue growth stays within 85% of the segment peak (20% in that band) and a bigger book no longer adds growth — that plateau is the data-driven target for headcount math. Segment avg PQR (prior quarter revenue per rep): $413K — the benchmark for whether a rep's book is revenue-heavy vs peers. Segment avg PCID: 107 accounts/rep — typical book size today; ideal PCID is the growth-optimal target, not the average. Current avg book (99) is below ideal — room to grow books toward the growth-optimal size before adding headcount. Too big = PCID or PQR above segment avg plus weak coverage or revenue below PQR; too little = below ideal PCID. Split/peel actions use ideal PCID as the target.</t>
         </is>
       </c>
     </row>
@@ -1764,12 +1857,27 @@
       </c>
       <c r="AW7" t="inlineStr">
         <is>
-          <t>Book health: 63 reps flagged too big, 11 too little (uneven books across the team). · PQR trend: Revenue is 22.0% above prior-quarter PQR (Hire signal from capacity model). · SBS whitespace: 385,800 unassigned accounts in this country × segment (~4,286 buildable books at ideal size). · Split-hire: Model suggests 22 new heads from 1,979 pooled PCIDs — Split-hire 22 new heads (1979 PCIDs pooled) · Market signals: opp pipeline plateaued, coverage ok. · FY26 book build: 46.8% of policy flags positive — room to improve book quality. · Recommended next step: Hire + build books from SBS.</t>
+          <t>Optimal book for this segment is 90 accounts/rep (81-100 band). We pick the largest book-size bucket where median revenue growth stays within 85% of the segment peak (20% in that band) and a bigger book no longer adds growth — that plateau is the data-driven target for headcount math. · Book health: 63 reps flagged too big, 11 too little (uneven books across the team). · PQR trend: Revenue is 22.0% above prior-quarter PQR (Hire signal from capacity model). · SBS whitespace: 385,800 unassigned accounts in this country × segment (~4,286 buildable books at ideal size). · Split-hire: Model suggests 22 new heads from 1,979 pooled PCIDs — Split-hire 22 new heads (1979 PCIDs pooled) · Market signals: opp pipeline plateaued, coverage ok. · FY26 book build: 46.8% of policy flags positive — room to improve book quality. · Recommended next step: Hire + build books from SBS.</t>
         </is>
       </c>
       <c r="AX7" t="inlineStr">
         <is>
-          <t>Under headcount by 20 reps (72 current vs 92 ideal). Avg book 115 vs ideal 90 — headcount is short but existing books are already above ideal; prioritize split/redistribution before pure hiring. Book health: 63 reps flagged too big, 11 too little (uneven books across the team). PQR trend: Revenue is 22.0% above prior-quarter PQR (Hire signal from capacity model). SBS whitespace: 385,800 unassigned accounts in this country × segment (~4,286 buildable books at ideal size). Split-hire: Model suggests 22 new heads from 1,979 pooled PCIDs — Split-hire 22 new heads (1979 PCIDs pooled) Market signals: opp pipeline plateaued, coverage ok. FY26 book build: 46.8% of policy flags positive — room to improve book quality. Recommended next step: Hire + build books from SBS.</t>
+          <t>Under headcount by 20 reps (72 current vs 92 ideal). Avg book 115 vs ideal 90 — headcount is short but existing books are already above ideal; prioritize split/redistribution before pure hiring. Optimal book for this segment is 90 accounts/rep (81-100 band). We pick the largest book-size bucket where median revenue growth stays within 85% of the segment peak (20% in that band) and a bigger book no longer adds growth — that plateau is the data-driven target for headcount math. Book health: 63 reps flagged too big, 11 too little (uneven books across the team). PQR trend: Revenue is 22.0% above prior-quarter PQR (Hire signal from capacity model). SBS whitespace: 385,800 unassigned accounts in this country × segment (~4,286 buildable books at ideal size). Split-hire: Model suggests 22 new heads from 1,979 pooled PCIDs — Split-hire 22 new heads (1979 PCIDs pooled) Market signals: opp pipeline plateaued, coverage ok. FY26 book build: 46.8% of policy flags positive — room to improve book quality. Recommended next step: Hire + build books from SBS.</t>
+        </is>
+      </c>
+      <c r="AY7" t="inlineStr">
+        <is>
+          <t>Optimal book for this segment is 90 accounts/rep (81-100 band). We pick the largest book-size bucket where median revenue growth stays within 85% of the segment peak (20% in that band) and a bigger book no longer adds growth — that plateau is the data-driven target for headcount math.</t>
+        </is>
+      </c>
+      <c r="AZ7" t="inlineStr">
+        <is>
+          <t>Segment avg PQR (prior quarter revenue per rep): $262K — the benchmark for whether a rep's book is revenue-heavy vs peers. · Segment avg PCID: 117 accounts/rep — typical book size today; ideal PCID is the growth-optimal target, not the average. · Current avg book (115) is above ideal — more accounts per rep can dilute coverage and drag growth; peel toward ideal PCID. · Opp pipeline plateaus around 100 accounts/rep — revenue per job peaks near this book size. · Coverage (impact calls/account) peaks near 150 accounts/rep — books larger than this tend to see fewer touches per account. · Too big = PCID or PQR above segment avg plus weak coverage or revenue below PQR; too little = below ideal PCID. Split/peel actions use ideal PCID as the target.</t>
+        </is>
+      </c>
+      <c r="BA7" t="inlineStr">
+        <is>
+          <t>Optimal book for this segment is 90 accounts/rep (81-100 band). We pick the largest book-size bucket where median revenue growth stays within 85% of the segment peak (20% in that band) and a bigger book no longer adds growth — that plateau is the data-driven target for headcount math. Segment avg PQR (prior quarter revenue per rep): $262K — the benchmark for whether a rep's book is revenue-heavy vs peers. Segment avg PCID: 117 accounts/rep — typical book size today; ideal PCID is the growth-optimal target, not the average. Current avg book (115) is above ideal — more accounts per rep can dilute coverage and drag growth; peel toward ideal PCID. Opp pipeline plateaus around 100 accounts/rep — revenue per job peaks near this book size. Coverage (impact calls/account) peaks near 150 accounts/rep — books larger than this tend to see fewer touches per account. Too big = PCID or PQR above segment avg plus weak coverage or revenue below PQR; too little = below ideal PCID. Split/peel actions use ideal PCID as the target.</t>
         </is>
       </c>
     </row>
@@ -1939,12 +2047,27 @@
       </c>
       <c r="AW8" t="inlineStr">
         <is>
-          <t>Book health: 19 reps flagged too big, 25 too little (uneven books across the team). · PQR trend: Revenue is 33.2% above prior-quarter PQR (Hire signal from capacity model). · SBS whitespace: 385,800 unassigned accounts in this country × segment (~25,720 buildable books at ideal size). · Split-hire: Model suggests 20 new heads from 304 pooled PCIDs — Split-hire 20 new heads (304 PCIDs pooled) · Market signals: opp pipeline plateaued, coverage ok. · Recommended next step: Hire + build books from SBS.</t>
+          <t>Optimal book for this segment is 15 accounts/rep (11-20 band). We pick the largest book-size bucket where median revenue growth stays within 85% of the segment peak (40% in that band) and a bigger book no longer adds growth — that plateau is the data-driven target for headcount math. · Book health: 19 reps flagged too big, 25 too little (uneven books across the team). · PQR trend: Revenue is 33.2% above prior-quarter PQR (Hire signal from capacity model). · SBS whitespace: 385,800 unassigned accounts in this country × segment (~25,720 buildable books at ideal size). · Split-hire: Model suggests 20 new heads from 304 pooled PCIDs — Split-hire 20 new heads (304 PCIDs pooled) · Market signals: opp pipeline plateaued, coverage ok. · Recommended next step: Hire + build books from SBS.</t>
         </is>
       </c>
       <c r="AX8" t="inlineStr">
         <is>
-          <t>Under headcount by 13 reps (49 current vs 62 ideal). Avg book 19 vs ideal 15 — headcount is short but existing books are already above ideal; prioritize split/redistribution before pure hiring. Book health: 19 reps flagged too big, 25 too little (uneven books across the team). PQR trend: Revenue is 33.2% above prior-quarter PQR (Hire signal from capacity model). SBS whitespace: 385,800 unassigned accounts in this country × segment (~25,720 buildable books at ideal size). Split-hire: Model suggests 20 new heads from 304 pooled PCIDs — Split-hire 20 new heads (304 PCIDs pooled) Market signals: opp pipeline plateaued, coverage ok. Recommended next step: Hire + build books from SBS.</t>
+          <t>Under headcount by 13 reps (49 current vs 62 ideal). Avg book 19 vs ideal 15 — headcount is short but existing books are already above ideal; prioritize split/redistribution before pure hiring. Optimal book for this segment is 15 accounts/rep (11-20 band). We pick the largest book-size bucket where median revenue growth stays within 85% of the segment peak (40% in that band) and a bigger book no longer adds growth — that plateau is the data-driven target for headcount math. Book health: 19 reps flagged too big, 25 too little (uneven books across the team). PQR trend: Revenue is 33.2% above prior-quarter PQR (Hire signal from capacity model). SBS whitespace: 385,800 unassigned accounts in this country × segment (~25,720 buildable books at ideal size). Split-hire: Model suggests 20 new heads from 304 pooled PCIDs — Split-hire 20 new heads (304 PCIDs pooled) Market signals: opp pipeline plateaued, coverage ok. Recommended next step: Hire + build books from SBS.</t>
+        </is>
+      </c>
+      <c r="AY8" t="inlineStr">
+        <is>
+          <t>Optimal book for this segment is 15 accounts/rep (11-20 band). We pick the largest book-size bucket where median revenue growth stays within 85% of the segment peak (40% in that band) and a bigger book no longer adds growth — that plateau is the data-driven target for headcount math.</t>
+        </is>
+      </c>
+      <c r="AZ8" t="inlineStr">
+        <is>
+          <t>Segment avg PQR (prior quarter revenue per rep): $114K — the benchmark for whether a rep's book is revenue-heavy vs peers. · Segment avg PCID: 19 accounts/rep — typical book size today; ideal PCID is the growth-optimal target, not the average. · Current avg book (19) is above ideal — more accounts per rep can dilute coverage and drag growth; peel toward ideal PCID. · Opp pipeline plateaus around 10 accounts/rep — revenue per job peaks near this book size. · Coverage (impact calls/account) peaks near 20 accounts/rep — books larger than this tend to see fewer touches per account. · Too big = PCID or PQR above segment avg plus weak coverage or revenue below PQR; too little = below ideal PCID. Split/peel actions use ideal PCID as the target.</t>
+        </is>
+      </c>
+      <c r="BA8" t="inlineStr">
+        <is>
+          <t>Optimal book for this segment is 15 accounts/rep (11-20 band). We pick the largest book-size bucket where median revenue growth stays within 85% of the segment peak (40% in that band) and a bigger book no longer adds growth — that plateau is the data-driven target for headcount math. Segment avg PQR (prior quarter revenue per rep): $114K — the benchmark for whether a rep's book is revenue-heavy vs peers. Segment avg PCID: 19 accounts/rep — typical book size today; ideal PCID is the growth-optimal target, not the average. Current avg book (19) is above ideal — more accounts per rep can dilute coverage and drag growth; peel toward ideal PCID. Opp pipeline plateaus around 10 accounts/rep — revenue per job peaks near this book size. Coverage (impact calls/account) peaks near 20 accounts/rep — books larger than this tend to see fewer touches per account. Too big = PCID or PQR above segment avg plus weak coverage or revenue below PQR; too little = below ideal PCID. Split/peel actions use ideal PCID as the target.</t>
         </is>
       </c>
     </row>
@@ -2114,17 +2237,32 @@
       </c>
       <c r="AW9" t="inlineStr">
         <is>
-          <t>Book health: 26 reps flagged too big, 27 too little (uneven books across the team). · PQR trend: Revenue is 32.9% above prior-quarter PQR (Hire signal from capacity model). · SBS whitespace: 157,800 unassigned accounts in this country × segment (~10,520 buildable books at ideal size). · Split-hire: Model suggests 26 new heads from 394 pooled PCIDs — Split-hire 26 new heads (394 PCIDs pooled) · Market signals: opp pipeline plateaued, coverage declining. · Recommended next step: Hire + build books from SBS.</t>
+          <t>Optimal book for this segment is 15 accounts/rep (11-20 band). We pick the largest book-size bucket where median revenue growth stays within 85% of the segment peak (40% in that band) and a bigger book no longer adds growth — that plateau is the data-driven target for headcount math. · Book health: 26 reps flagged too big, 27 too little (uneven books across the team). · PQR trend: Revenue is 32.9% above prior-quarter PQR (Hire signal from capacity model). · SBS whitespace: 157,800 unassigned accounts in this country × segment (~10,520 buildable books at ideal size). · Split-hire: Model suggests 26 new heads from 394 pooled PCIDs — Split-hire 26 new heads (394 PCIDs pooled) · Market signals: opp pipeline plateaued, coverage declining. · Recommended next step: Hire + build books from SBS.</t>
         </is>
       </c>
       <c r="AX9" t="inlineStr">
         <is>
-          <t>Under headcount by 24 reps (59 current vs 83 ideal). Avg book 21 vs ideal 15 — headcount is short but existing books are already above ideal; prioritize split/redistribution before pure hiring. Book health: 26 reps flagged too big, 27 too little (uneven books across the team). PQR trend: Revenue is 32.9% above prior-quarter PQR (Hire signal from capacity model). SBS whitespace: 157,800 unassigned accounts in this country × segment (~10,520 buildable books at ideal size). Split-hire: Model suggests 26 new heads from 394 pooled PCIDs — Split-hire 26 new heads (394 PCIDs pooled) Market signals: opp pipeline plateaued, coverage declining. Recommended next step: Hire + build books from SBS.</t>
+          <t>Under headcount by 24 reps (59 current vs 83 ideal). Avg book 21 vs ideal 15 — headcount is short but existing books are already above ideal; prioritize split/redistribution before pure hiring. Optimal book for this segment is 15 accounts/rep (11-20 band). We pick the largest book-size bucket where median revenue growth stays within 85% of the segment peak (40% in that band) and a bigger book no longer adds growth — that plateau is the data-driven target for headcount math. Book health: 26 reps flagged too big, 27 too little (uneven books across the team). PQR trend: Revenue is 32.9% above prior-quarter PQR (Hire signal from capacity model). SBS whitespace: 157,800 unassigned accounts in this country × segment (~10,520 buildable books at ideal size). Split-hire: Model suggests 26 new heads from 394 pooled PCIDs — Split-hire 26 new heads (394 PCIDs pooled) Market signals: opp pipeline plateaued, coverage declining. Recommended next step: Hire + build books from SBS.</t>
+        </is>
+      </c>
+      <c r="AY9" t="inlineStr">
+        <is>
+          <t>Optimal book for this segment is 15 accounts/rep (11-20 band). We pick the largest book-size bucket where median revenue growth stays within 85% of the segment peak (40% in that band) and a bigger book no longer adds growth — that plateau is the data-driven target for headcount math.</t>
+        </is>
+      </c>
+      <c r="AZ9" t="inlineStr">
+        <is>
+          <t>Segment avg PQR (prior quarter revenue per rep): $65K — the benchmark for whether a rep's book is revenue-heavy vs peers. · Segment avg PCID: 20 accounts/rep — typical book size today; ideal PCID is the growth-optimal target, not the average. · Current avg book (21) is above ideal — more accounts per rep can dilute coverage and drag growth; peel toward ideal PCID. · Opp pipeline plateaus around 10 accounts/rep — revenue per job peaks near this book size. · Coverage (impact calls/account) peaks near 10 accounts/rep — books larger than this tend to see fewer touches per account. · Too big = PCID or PQR above segment avg plus weak coverage or revenue below PQR; too little = below ideal PCID. Split/peel actions use ideal PCID as the target.</t>
+        </is>
+      </c>
+      <c r="BA9" t="inlineStr">
+        <is>
+          <t>Optimal book for this segment is 15 accounts/rep (11-20 band). We pick the largest book-size bucket where median revenue growth stays within 85% of the segment peak (40% in that band) and a bigger book no longer adds growth — that plateau is the data-driven target for headcount math. Segment avg PQR (prior quarter revenue per rep): $65K — the benchmark for whether a rep's book is revenue-heavy vs peers. Segment avg PCID: 20 accounts/rep — typical book size today; ideal PCID is the growth-optimal target, not the average. Current avg book (21) is above ideal — more accounts per rep can dilute coverage and drag growth; peel toward ideal PCID. Opp pipeline plateaus around 10 accounts/rep — revenue per job peaks near this book size. Coverage (impact calls/account) peaks near 10 accounts/rep — books larger than this tend to see fewer touches per account. Too big = PCID or PQR above segment avg plus weak coverage or revenue below PQR; too little = below ideal PCID. Split/peel actions use ideal PCID as the target.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AX9"/>
+  <autoFilter ref="A1:BA9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -105333,7 +105471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:N9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -105342,9 +105480,14 @@
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="72" customWidth="1" min="5" max="5"/>
     <col width="88" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
-    <col width="19" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="31" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="17" customWidth="1" min="10" max="10"/>
+    <col width="21" customWidth="1" min="11" max="11"/>
+    <col width="15" customWidth="1" min="12" max="12"/>
+    <col width="19" customWidth="1" min="13" max="13"/>
+    <col width="20" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -105380,15 +105523,40 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>Optimal book — why</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Optimal book — full rationale</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Ideal PCID</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Ideal book size</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Segment avg PQR ($)</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
           <t>Headcount gap</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>HC recommendation</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Recommended action</t>
         </is>
@@ -105422,18 +105590,37 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Book health: 77 reps flagged too big, 1 too little (uneven books across the team). · PQR trend: Revenue is 17.6% above prior-quarter PQR (Hire signal from capacity model). · SBS whitespace: 1,908,879 unassigned accounts in this country × segment (~21,209 buildable books at ideal size). · Split-hire: Model suggests 85 new heads from 7,699 pooled PCIDs — Split-hire 85 new heads (7699 PCIDs pooled) · Market signals: opp pipeline plateaued, coverage ok. · FY26 book build: 46.3% of policy flags positive — room to improve book quality. · Recommended next step: Hire + build books from SBS.</t>
-        </is>
-      </c>
-      <c r="G2" t="n">
+          <t>Optimal book for this segment is 90 accounts/rep (81-100 band). We pick the largest book-size bucket where median revenue growth stays within 85% of the segment peak (20% in that band) and a bigger book no longer adds growth — that plateau is the data-driven target for headcount math. · Book health: 77 reps flagged too big, 1 too little (uneven books across the team). · PQR trend: Revenue is 17.6% above prior-quarter PQR (Hire signal from capacity model). · SBS whitespace: 1,908,879 unassigned accounts in this country × segment (~21,209 buildable books at ideal size). · Split-hire: Model suggests 85 new heads from 7,699 pooled PCIDs — Split-hire 85 new heads (7699 PCIDs pooled) · Market signals: opp pipeline plateaued, coverage ok. · FY26 book build: 46.3% of policy flags positive — room to improve book quality. · Recommended next step: Hire + build books from SBS.</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Optimal book for this segment is 90 accounts/rep (81-100 band). We pick the largest book-size bucket where median revenue growth stays within 85% of the segment peak (20% in that band) and a bigger book no longer adds growth — that plateau is the data-driven target for headcount math.</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Optimal book for this segment is 90 accounts/rep (81-100 band). We pick the largest book-size bucket where median revenue growth stays within 85% of the segment peak (20% in that band) and a bigger book no longer adds growth — that plateau is the data-driven target for headcount math. Segment avg PQR (prior quarter revenue per rep): $407K — the benchmark for whether a rep's book is revenue-heavy vs peers. Segment avg PCID: 125 accounts/rep — typical book size today; ideal PCID is the growth-optimal target, not the average. Current avg book (127) is above ideal — more accounts per rep can dilute coverage and drag growth; peel toward ideal PCID. Opp pipeline plateaus around 100 accounts/rep — revenue per job peaks near this book size. Coverage (impact calls/account) peaks near 100 accounts/rep — books larger than this tend to see fewer touches per account. Too big = PCID or PQR above segment avg plus weak coverage or revenue below PQR; too little = below ideal PCID. Split/peel actions use ideal PCID as the target.</t>
+        </is>
+      </c>
+      <c r="I2" t="n">
+        <v>90</v>
+      </c>
+      <c r="J2" t="n">
+        <v>90</v>
+      </c>
+      <c r="K2" t="n">
+        <v>406667</v>
+      </c>
+      <c r="L2" t="n">
         <v>-93</v>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>Hire</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>Hire + build books from SBS</t>
         </is>
@@ -105467,18 +105654,37 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Book health: 81 reps flagged too big, 204 too little (uneven books across the team). · PQR trend: Revenue is 20.5% above prior-quarter PQR (Optimize signal from capacity model). · SBS whitespace: 1,908,879 unassigned accounts in this country × segment (~32,911 buildable books at ideal size). · Book action: Redistribute internally (too big → too little). · Market signals: opp pipeline growing, coverage ok. · FY26 book build: 49.1% of policy flags positive — room to improve book quality. · Recommended next step: Optimize HC.</t>
-        </is>
-      </c>
-      <c r="G3" t="n">
+          <t>Optimal book for this segment is 58 accounts/rep (51-65 band). We pick the largest book-size bucket where median revenue growth stays within 85% of the segment peak (20% in that band) and a bigger book no longer adds growth — that plateau is the data-driven target for headcount math. · Book health: 81 reps flagged too big, 204 too little (uneven books across the team). · PQR trend: Revenue is 20.5% above prior-quarter PQR (Optimize signal from capacity model). · SBS whitespace: 1,908,879 unassigned accounts in this country × segment (~32,911 buildable books at ideal size). · Book action: Redistribute internally (too big → too little). · Market signals: opp pipeline growing, coverage ok. · FY26 book build: 49.1% of policy flags positive — room to improve book quality. · Recommended next step: Optimize HC.</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Optimal book for this segment is 58 accounts/rep (51-65 band). We pick the largest book-size bucket where median revenue growth stays within 85% of the segment peak (20% in that band) and a bigger book no longer adds growth — that plateau is the data-driven target for headcount math.</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Optimal book for this segment is 58 accounts/rep (51-65 band). We pick the largest book-size bucket where median revenue growth stays within 85% of the segment peak (20% in that band) and a bigger book no longer adds growth — that plateau is the data-driven target for headcount math. Segment avg PQR (prior quarter revenue per rep): $415K — the benchmark for whether a rep's book is revenue-heavy vs peers. Segment avg PCID: 40 accounts/rep — typical book size today; ideal PCID is the growth-optimal target, not the average. Current avg book (39) is below ideal — room to grow books toward the growth-optimal size before adding headcount. Opp pipeline still growing around 50 accounts/rep — revenue per job peaks near this book size. Coverage (impact calls/account) peaks near 65 accounts/rep — books larger than this tend to see fewer touches per account. Too big = PCID or PQR above segment avg plus weak coverage or revenue below PQR; too little = below ideal PCID. Split/peel actions use ideal PCID as the target.</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>58</v>
+      </c>
+      <c r="J3" t="n">
+        <v>58</v>
+      </c>
+      <c r="K3" t="n">
+        <v>414548</v>
+      </c>
+      <c r="L3" t="n">
         <v>68</v>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>Optimize</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>Optimize HC</t>
         </is>
@@ -105512,18 +105718,37 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Book health: 108 reps flagged too big, 57 too little (uneven books across the team). · PQR trend: Revenue is 29.0% above prior-quarter PQR (Hire signal from capacity model). · SBS whitespace: 1,908,879 unassigned accounts in this country × segment (~381,775 buildable books at ideal size). · Split-hire: Model suggests 473 new heads from 2,369 pooled PCIDs — Split-hire 473 new heads (2369 PCIDs pooled) · Market signals: opp pipeline growing, coverage ok. · Recommended next step: Hire + build books from SBS.</t>
-        </is>
-      </c>
-      <c r="G4" t="n">
+          <t>Optimal book for this segment is 5 accounts/rep (1-10 band). We pick the largest book-size bucket where median revenue growth stays within 85% of the segment peak (23% in that band) and a bigger book no longer adds growth — that plateau is the data-driven target for headcount math. · Book health: 108 reps flagged too big, 57 too little (uneven books across the team). · PQR trend: Revenue is 29.0% above prior-quarter PQR (Hire signal from capacity model). · SBS whitespace: 1,908,879 unassigned accounts in this country × segment (~381,775 buildable books at ideal size). · Split-hire: Model suggests 473 new heads from 2,369 pooled PCIDs — Split-hire 473 new heads (2369 PCIDs pooled) · Market signals: opp pipeline growing, coverage ok. · Recommended next step: Hire + build books from SBS.</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Optimal book for this segment is 5 accounts/rep (1-10 band). We pick the largest book-size bucket where median revenue growth stays within 85% of the segment peak (23% in that band) and a bigger book no longer adds growth — that plateau is the data-driven target for headcount math.</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Optimal book for this segment is 5 accounts/rep (1-10 band). We pick the largest book-size bucket where median revenue growth stays within 85% of the segment peak (23% in that band) and a bigger book no longer adds growth — that plateau is the data-driven target for headcount math. Segment avg PQR (prior quarter revenue per rep): $249K — the benchmark for whether a rep's book is revenue-heavy vs peers. Segment avg PCID: 16 accounts/rep — typical book size today; ideal PCID is the growth-optimal target, not the average. Current avg book (16) is above ideal — more accounts per rep can dilute coverage and drag growth; peel toward ideal PCID. Opp pipeline still growing around 50 accounts/rep — revenue per job peaks near this book size. Coverage (impact calls/account) peaks near 50 accounts/rep — books larger than this tend to see fewer touches per account. Too big = PCID or PQR above segment avg plus weak coverage or revenue below PQR; too little = below ideal PCID. Split/peel actions use ideal PCID as the target.</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>5</v>
+      </c>
+      <c r="J4" t="n">
+        <v>5</v>
+      </c>
+      <c r="K4" t="n">
+        <v>248956</v>
+      </c>
+      <c r="L4" t="n">
         <v>-520</v>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>Hire</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>Hire + build books from SBS</t>
         </is>
@@ -105557,18 +105782,37 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Book health: 39 reps flagged too big, 3 too little (uneven books across the team). · PQR trend: Revenue is 17.7% above prior-quarter PQR (Hold signal from capacity model). · SBS whitespace: 1,908,879 unassigned accounts in this country × segment (~32,911 buildable books at ideal size). · Split-hire: Model suggests 3 new heads from 199 pooled PCIDs — Split-hire 3 new heads (199 PCIDs pooled) · Market signals: opp pipeline growing, coverage ok. · FY26 book build: 47.4% of policy flags positive — room to improve book quality. · Recommended next step: Improve FY26 book build score.</t>
-        </is>
-      </c>
-      <c r="G5" t="n">
+          <t>Optimal book for this segment is 58 accounts/rep (51-65 band). We pick the largest book-size bucket where median revenue growth stays within 85% of the segment peak (20% in that band) and a bigger book no longer adds growth — that plateau is the data-driven target for headcount math. · Book health: 39 reps flagged too big, 3 too little (uneven books across the team). · PQR trend: Revenue is 17.7% above prior-quarter PQR (Hold signal from capacity model). · SBS whitespace: 1,908,879 unassigned accounts in this country × segment (~32,911 buildable books at ideal size). · Split-hire: Model suggests 3 new heads from 199 pooled PCIDs — Split-hire 3 new heads (199 PCIDs pooled) · Market signals: opp pipeline growing, coverage ok. · FY26 book build: 47.4% of policy flags positive — room to improve book quality. · Recommended next step: Improve FY26 book build score.</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Optimal book for this segment is 58 accounts/rep (51-65 band). We pick the largest book-size bucket where median revenue growth stays within 85% of the segment peak (20% in that band) and a bigger book no longer adds growth — that plateau is the data-driven target for headcount math.</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Optimal book for this segment is 58 accounts/rep (51-65 band). We pick the largest book-size bucket where median revenue growth stays within 85% of the segment peak (20% in that band) and a bigger book no longer adds growth — that plateau is the data-driven target for headcount math. Segment avg PQR (prior quarter revenue per rep): $387K — the benchmark for whether a rep's book is revenue-heavy vs peers. Segment avg PCID: 61 accounts/rep — typical book size today; ideal PCID is the growth-optimal target, not the average. Opp pipeline still growing around 65 accounts/rep — revenue per job peaks near this book size. Coverage (impact calls/account) peaks near 65 accounts/rep — books larger than this tend to see fewer touches per account. Too big = PCID or PQR above segment avg plus weak coverage or revenue below PQR; too little = below ideal PCID. Split/peel actions use ideal PCID as the target.</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>58</v>
+      </c>
+      <c r="J5" t="n">
+        <v>58</v>
+      </c>
+      <c r="K5" t="n">
+        <v>387103</v>
+      </c>
+      <c r="L5" t="n">
         <v>-7</v>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="M5" t="inlineStr">
         <is>
           <t>Hold</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="N5" t="inlineStr">
         <is>
           <t>Improve FY26 book build score</t>
         </is>
@@ -105602,18 +105846,37 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Book health: 69 reps flagged too big, 72 too little (uneven books across the team). · PQR trend: Revenue is 16.2% above prior-quarter PQR (Optimize signal from capacity model). · SBS whitespace: 1,908,879 unassigned accounts in this country × segment (~13,832 buildable books at ideal size). · Split-hire: Model suggests 2 new heads from 306 pooled PCIDs — Split-hire 2 new heads (306 PCIDs pooled) · Market signals: opp pipeline unknown, coverage ok. · FY26 book build: 45.0% of policy flags positive — room to improve book quality. · Recommended next step: Optimize HC.</t>
-        </is>
-      </c>
-      <c r="G6" t="n">
+          <t>Optimal book for this segment is 138 accounts/rep (126-150 band). We pick the largest book-size bucket where median revenue growth stays within 85% of the segment peak (20% in that band) and a bigger book no longer adds growth — that plateau is the data-driven target for headcount math. · Book health: 69 reps flagged too big, 72 too little (uneven books across the team). · PQR trend: Revenue is 16.2% above prior-quarter PQR (Optimize signal from capacity model). · SBS whitespace: 1,908,879 unassigned accounts in this country × segment (~13,832 buildable books at ideal size). · Split-hire: Model suggests 2 new heads from 306 pooled PCIDs — Split-hire 2 new heads (306 PCIDs pooled) · Market signals: opp pipeline unknown, coverage ok. · FY26 book build: 45.0% of policy flags positive — room to improve book quality. · Recommended next step: Optimize HC.</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Optimal book for this segment is 138 accounts/rep (126-150 band). We pick the largest book-size bucket where median revenue growth stays within 85% of the segment peak (20% in that band) and a bigger book no longer adds growth — that plateau is the data-driven target for headcount math.</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Optimal book for this segment is 138 accounts/rep (126-150 band). We pick the largest book-size bucket where median revenue growth stays within 85% of the segment peak (20% in that band) and a bigger book no longer adds growth — that plateau is the data-driven target for headcount math. Segment avg PQR (prior quarter revenue per rep): $413K — the benchmark for whether a rep's book is revenue-heavy vs peers. Segment avg PCID: 107 accounts/rep — typical book size today; ideal PCID is the growth-optimal target, not the average. Current avg book (99) is below ideal — room to grow books toward the growth-optimal size before adding headcount. Too big = PCID or PQR above segment avg plus weak coverage or revenue below PQR; too little = below ideal PCID. Split/peel actions use ideal PCID as the target.</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>138</v>
+      </c>
+      <c r="J6" t="n">
+        <v>138</v>
+      </c>
+      <c r="K6" t="n">
+        <v>412656</v>
+      </c>
+      <c r="L6" t="n">
         <v>31</v>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="M6" t="inlineStr">
         <is>
           <t>Optimize</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="N6" t="inlineStr">
         <is>
           <t>Optimize HC</t>
         </is>
@@ -105647,18 +105910,37 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Book health: 63 reps flagged too big, 11 too little (uneven books across the team). · PQR trend: Revenue is 22.0% above prior-quarter PQR (Hire signal from capacity model). · SBS whitespace: 385,800 unassigned accounts in this country × segment (~4,286 buildable books at ideal size). · Split-hire: Model suggests 22 new heads from 1,979 pooled PCIDs — Split-hire 22 new heads (1979 PCIDs pooled) · Market signals: opp pipeline plateaued, coverage ok. · FY26 book build: 46.8% of policy flags positive — room to improve book quality. · Recommended next step: Hire + build books from SBS.</t>
-        </is>
-      </c>
-      <c r="G7" t="n">
+          <t>Optimal book for this segment is 90 accounts/rep (81-100 band). We pick the largest book-size bucket where median revenue growth stays within 85% of the segment peak (20% in that band) and a bigger book no longer adds growth — that plateau is the data-driven target for headcount math. · Book health: 63 reps flagged too big, 11 too little (uneven books across the team). · PQR trend: Revenue is 22.0% above prior-quarter PQR (Hire signal from capacity model). · SBS whitespace: 385,800 unassigned accounts in this country × segment (~4,286 buildable books at ideal size). · Split-hire: Model suggests 22 new heads from 1,979 pooled PCIDs — Split-hire 22 new heads (1979 PCIDs pooled) · Market signals: opp pipeline plateaued, coverage ok. · FY26 book build: 46.8% of policy flags positive — room to improve book quality. · Recommended next step: Hire + build books from SBS.</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Optimal book for this segment is 90 accounts/rep (81-100 band). We pick the largest book-size bucket where median revenue growth stays within 85% of the segment peak (20% in that band) and a bigger book no longer adds growth — that plateau is the data-driven target for headcount math.</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Optimal book for this segment is 90 accounts/rep (81-100 band). We pick the largest book-size bucket where median revenue growth stays within 85% of the segment peak (20% in that band) and a bigger book no longer adds growth — that plateau is the data-driven target for headcount math. Segment avg PQR (prior quarter revenue per rep): $262K — the benchmark for whether a rep's book is revenue-heavy vs peers. Segment avg PCID: 117 accounts/rep — typical book size today; ideal PCID is the growth-optimal target, not the average. Current avg book (115) is above ideal — more accounts per rep can dilute coverage and drag growth; peel toward ideal PCID. Opp pipeline plateaus around 100 accounts/rep — revenue per job peaks near this book size. Coverage (impact calls/account) peaks near 150 accounts/rep — books larger than this tend to see fewer touches per account. Too big = PCID or PQR above segment avg plus weak coverage or revenue below PQR; too little = below ideal PCID. Split/peel actions use ideal PCID as the target.</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>90</v>
+      </c>
+      <c r="J7" t="n">
+        <v>90</v>
+      </c>
+      <c r="K7" t="n">
+        <v>262368</v>
+      </c>
+      <c r="L7" t="n">
         <v>-20</v>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="M7" t="inlineStr">
         <is>
           <t>Hire</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="N7" t="inlineStr">
         <is>
           <t>Hire + build books from SBS</t>
         </is>
@@ -105692,18 +105974,37 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Book health: 19 reps flagged too big, 25 too little (uneven books across the team). · PQR trend: Revenue is 33.2% above prior-quarter PQR (Hire signal from capacity model). · SBS whitespace: 385,800 unassigned accounts in this country × segment (~25,720 buildable books at ideal size). · Split-hire: Model suggests 20 new heads from 304 pooled PCIDs — Split-hire 20 new heads (304 PCIDs pooled) · Market signals: opp pipeline plateaued, coverage ok. · Recommended next step: Hire + build books from SBS.</t>
-        </is>
-      </c>
-      <c r="G8" t="n">
+          <t>Optimal book for this segment is 15 accounts/rep (11-20 band). We pick the largest book-size bucket where median revenue growth stays within 85% of the segment peak (40% in that band) and a bigger book no longer adds growth — that plateau is the data-driven target for headcount math. · Book health: 19 reps flagged too big, 25 too little (uneven books across the team). · PQR trend: Revenue is 33.2% above prior-quarter PQR (Hire signal from capacity model). · SBS whitespace: 385,800 unassigned accounts in this country × segment (~25,720 buildable books at ideal size). · Split-hire: Model suggests 20 new heads from 304 pooled PCIDs — Split-hire 20 new heads (304 PCIDs pooled) · Market signals: opp pipeline plateaued, coverage ok. · Recommended next step: Hire + build books from SBS.</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Optimal book for this segment is 15 accounts/rep (11-20 band). We pick the largest book-size bucket where median revenue growth stays within 85% of the segment peak (40% in that band) and a bigger book no longer adds growth — that plateau is the data-driven target for headcount math.</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Optimal book for this segment is 15 accounts/rep (11-20 band). We pick the largest book-size bucket where median revenue growth stays within 85% of the segment peak (40% in that band) and a bigger book no longer adds growth — that plateau is the data-driven target for headcount math. Segment avg PQR (prior quarter revenue per rep): $114K — the benchmark for whether a rep's book is revenue-heavy vs peers. Segment avg PCID: 19 accounts/rep — typical book size today; ideal PCID is the growth-optimal target, not the average. Current avg book (19) is above ideal — more accounts per rep can dilute coverage and drag growth; peel toward ideal PCID. Opp pipeline plateaus around 10 accounts/rep — revenue per job peaks near this book size. Coverage (impact calls/account) peaks near 20 accounts/rep — books larger than this tend to see fewer touches per account. Too big = PCID or PQR above segment avg plus weak coverage or revenue below PQR; too little = below ideal PCID. Split/peel actions use ideal PCID as the target.</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>15</v>
+      </c>
+      <c r="J8" t="n">
+        <v>15</v>
+      </c>
+      <c r="K8" t="n">
+        <v>113728</v>
+      </c>
+      <c r="L8" t="n">
         <v>-13</v>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="M8" t="inlineStr">
         <is>
           <t>Hire</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="N8" t="inlineStr">
         <is>
           <t>Hire + build books from SBS</t>
         </is>
@@ -105737,25 +106038,44 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Book health: 26 reps flagged too big, 27 too little (uneven books across the team). · PQR trend: Revenue is 32.9% above prior-quarter PQR (Hire signal from capacity model). · SBS whitespace: 157,800 unassigned accounts in this country × segment (~10,520 buildable books at ideal size). · Split-hire: Model suggests 26 new heads from 394 pooled PCIDs — Split-hire 26 new heads (394 PCIDs pooled) · Market signals: opp pipeline plateaued, coverage declining. · Recommended next step: Hire + build books from SBS.</t>
-        </is>
-      </c>
-      <c r="G9" t="n">
+          <t>Optimal book for this segment is 15 accounts/rep (11-20 band). We pick the largest book-size bucket where median revenue growth stays within 85% of the segment peak (40% in that band) and a bigger book no longer adds growth — that plateau is the data-driven target for headcount math. · Book health: 26 reps flagged too big, 27 too little (uneven books across the team). · PQR trend: Revenue is 32.9% above prior-quarter PQR (Hire signal from capacity model). · SBS whitespace: 157,800 unassigned accounts in this country × segment (~10,520 buildable books at ideal size). · Split-hire: Model suggests 26 new heads from 394 pooled PCIDs — Split-hire 26 new heads (394 PCIDs pooled) · Market signals: opp pipeline plateaued, coverage declining. · Recommended next step: Hire + build books from SBS.</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Optimal book for this segment is 15 accounts/rep (11-20 band). We pick the largest book-size bucket where median revenue growth stays within 85% of the segment peak (40% in that band) and a bigger book no longer adds growth — that plateau is the data-driven target for headcount math.</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Optimal book for this segment is 15 accounts/rep (11-20 band). We pick the largest book-size bucket where median revenue growth stays within 85% of the segment peak (40% in that band) and a bigger book no longer adds growth — that plateau is the data-driven target for headcount math. Segment avg PQR (prior quarter revenue per rep): $65K — the benchmark for whether a rep's book is revenue-heavy vs peers. Segment avg PCID: 20 accounts/rep — typical book size today; ideal PCID is the growth-optimal target, not the average. Current avg book (21) is above ideal — more accounts per rep can dilute coverage and drag growth; peel toward ideal PCID. Opp pipeline plateaus around 10 accounts/rep — revenue per job peaks near this book size. Coverage (impact calls/account) peaks near 10 accounts/rep — books larger than this tend to see fewer touches per account. Too big = PCID or PQR above segment avg plus weak coverage or revenue below PQR; too little = below ideal PCID. Split/peel actions use ideal PCID as the target.</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>15</v>
+      </c>
+      <c r="J9" t="n">
+        <v>15</v>
+      </c>
+      <c r="K9" t="n">
+        <v>65371</v>
+      </c>
+      <c r="L9" t="n">
         <v>-24</v>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="M9" t="inlineStr">
         <is>
           <t>Hire</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="N9" t="inlineStr">
         <is>
           <t>Hire + build books from SBS</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I9"/>
+  <autoFilter ref="A1:N9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -105901,7 +106221,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-28</t>
         </is>
       </c>
     </row>

</xml_diff>